<commit_message>
in-house / subcontract column
</commit_message>
<xml_diff>
--- a/quote-builder/Riverbend-Q900142-Costing.xlsx
+++ b/quote-builder/Riverbend-Q900142-Costing.xlsx
@@ -54,7 +54,7 @@
       <sz val="10.5"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -81,6 +81,11 @@
         <fgColor rgb="00E8F0FB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6F4EC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -94,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -122,6 +127,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -834,19 +840,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J66"/>
+  <dimension ref="A1:K66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="32" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -872,30 +879,35 @@
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
+          <t>Who does it</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Unit cost</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Margin</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -920,6 +932,7 @@
       <c r="H2" s="6" t="n"/>
       <c r="I2" s="6" t="n"/>
       <c r="J2" s="6" t="n"/>
+      <c r="K2" s="6" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n"/>
@@ -938,23 +951,23 @@
           <t>RFQ</t>
         </is>
       </c>
-      <c r="E3" s="7" t="n">
+      <c r="F3" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="G3" s="9" t="n"/>
-      <c r="H3" s="10" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I3" s="9">
-        <f>IFERROR($E3*$G3,"")</f>
-        <v/>
-      </c>
-      <c r="J3" s="11" t="inlineStr">
+      <c r="H3" s="9" t="n"/>
+      <c r="I3" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J3" s="9">
+        <f>IFERROR($F3*$H3,"")</f>
+        <v/>
+      </c>
+      <c r="K3" s="11" t="inlineStr">
         <is>
           <t>90 kW each · IE5 VSD</t>
         </is>
@@ -979,6 +992,7 @@
       <c r="H4" s="6" t="n"/>
       <c r="I4" s="6" t="n"/>
       <c r="J4" s="6" t="n"/>
+      <c r="K4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n"/>
@@ -997,23 +1011,23 @@
           <t>RFQ</t>
         </is>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="F5" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="G5" s="9" t="n"/>
-      <c r="H5" s="10" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I5" s="9">
-        <f>IFERROR($E5*$G5,"")</f>
-        <v/>
-      </c>
-      <c r="J5" s="11" t="inlineStr">
+      <c r="H5" s="9" t="n"/>
+      <c r="I5" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J5" s="9">
+        <f>IFERROR($F5*$H5,"")</f>
+        <v/>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
         <is>
           <t>620 kWR each · EC Fan Supply</t>
         </is>
@@ -1038,6 +1052,7 @@
       <c r="H6" s="6" t="n"/>
       <c r="I6" s="6" t="n"/>
       <c r="J6" s="6" t="n"/>
+      <c r="K6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n"/>
@@ -1056,23 +1071,23 @@
           <t>RFQ</t>
         </is>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="F7" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="G7" s="9" t="n"/>
-      <c r="H7" s="10" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I7" s="9">
-        <f>IFERROR($E7*$G7,"")</f>
-        <v/>
-      </c>
-      <c r="J7" s="11" t="inlineStr">
+      <c r="H7" s="9" t="n"/>
+      <c r="I7" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J7" s="9">
+        <f>IFERROR($F7*$H7,"")</f>
+        <v/>
+      </c>
+      <c r="K7" s="11" t="inlineStr">
         <is>
           <t>520 kWR each · no starter shown</t>
         </is>
@@ -1097,6 +1112,7 @@
       <c r="H8" s="6" t="n"/>
       <c r="I8" s="6" t="n"/>
       <c r="J8" s="6" t="n"/>
+      <c r="K8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n"/>
@@ -1115,23 +1131,23 @@
           <t>RFQ</t>
         </is>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="F9" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="G9" s="7" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="G9" s="9" t="n"/>
-      <c r="H9" s="10" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I9" s="9">
-        <f>IFERROR($E9*$G9,"")</f>
-        <v/>
-      </c>
-      <c r="J9" s="11" t="inlineStr">
+      <c r="H9" s="9" t="n"/>
+      <c r="I9" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J9" s="9">
+        <f>IFERROR($F9*$H9,"")</f>
+        <v/>
+      </c>
+      <c r="K9" s="11" t="inlineStr">
         <is>
           <t>15 kW each · VSD</t>
         </is>
@@ -1154,23 +1170,23 @@
           <t>RFQ</t>
         </is>
       </c>
-      <c r="E10" s="7" t="n">
+      <c r="F10" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="G10" s="9" t="n"/>
-      <c r="H10" s="10" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I10" s="9">
-        <f>IFERROR($E10*$G10,"")</f>
-        <v/>
-      </c>
-      <c r="J10" s="11" t="inlineStr">
+      <c r="H10" s="9" t="n"/>
+      <c r="I10" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J10" s="9">
+        <f>IFERROR($F10*$H10,"")</f>
+        <v/>
+      </c>
+      <c r="K10" s="11" t="inlineStr">
         <is>
           <t>4 kW each · VSD</t>
         </is>
@@ -1195,6 +1211,7 @@
       <c r="H11" s="6" t="n"/>
       <c r="I11" s="6" t="n"/>
       <c r="J11" s="6" t="n"/>
+      <c r="K11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n"/>
@@ -1213,23 +1230,23 @@
           <t>RFQ</t>
         </is>
       </c>
-      <c r="E12" s="7" t="n">
+      <c r="F12" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="G12" s="9" t="n"/>
-      <c r="H12" s="10" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I12" s="9">
-        <f>IFERROR($E12*$G12,"")</f>
-        <v/>
-      </c>
-      <c r="J12" s="11" t="inlineStr">
+      <c r="H12" s="9" t="n"/>
+      <c r="I12" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J12" s="9">
+        <f>IFERROR($F12*$H12,"")</f>
+        <v/>
+      </c>
+      <c r="K12" s="11" t="inlineStr">
         <is>
           <t>55 kWR each · EC Fan Supply</t>
         </is>
@@ -1254,6 +1271,7 @@
       <c r="H13" s="6" t="n"/>
       <c r="I13" s="6" t="n"/>
       <c r="J13" s="6" t="n"/>
+      <c r="K13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
@@ -1272,23 +1290,23 @@
           <t>RFQ</t>
         </is>
       </c>
-      <c r="E14" s="7" t="n">
+      <c r="F14" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="G14" s="9" t="n"/>
-      <c r="H14" s="10" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I14" s="9">
-        <f>IFERROR($E14*$G14,"")</f>
-        <v/>
-      </c>
-      <c r="J14" s="11" t="inlineStr">
+      <c r="H14" s="9" t="n"/>
+      <c r="I14" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J14" s="9">
+        <f>IFERROR($F14*$H14,"")</f>
+        <v/>
+      </c>
+      <c r="K14" s="11" t="inlineStr">
         <is>
           <t>10 × 50TE on the P&amp;ID</t>
         </is>
@@ -1311,23 +1329,23 @@
           <t>RULE</t>
         </is>
       </c>
-      <c r="E15" s="12" t="n">
+      <c r="F15" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="F15" s="12" t="inlineStr">
+      <c r="G15" s="12" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="G15" s="14" t="n"/>
-      <c r="H15" s="15" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I15" s="14">
-        <f>IFERROR($E15*$G15,"")</f>
-        <v/>
-      </c>
-      <c r="J15" s="16" t="inlineStr">
+      <c r="H15" s="14" t="n"/>
+      <c r="I15" s="15" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J15" s="14">
+        <f>IFERROR($F15*$H15,"")</f>
+        <v/>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
         <is>
           <t>rule: 1 per 50TE connection</t>
         </is>
@@ -1350,23 +1368,23 @@
           <t>RULE</t>
         </is>
       </c>
-      <c r="E16" s="12" t="n">
+      <c r="F16" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="F16" s="12" t="inlineStr">
+      <c r="G16" s="12" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="G16" s="14" t="n"/>
-      <c r="H16" s="15" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I16" s="14">
-        <f>IFERROR($E16*$G16,"")</f>
-        <v/>
-      </c>
-      <c r="J16" s="16" t="inlineStr">
+      <c r="H16" s="14" t="n"/>
+      <c r="I16" s="15" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J16" s="14">
+        <f>IFERROR($F16*$H16,"")</f>
+        <v/>
+      </c>
+      <c r="K16" s="16" t="inlineStr">
         <is>
           <t>rule: 1 per 50TE connection</t>
         </is>
@@ -1389,23 +1407,23 @@
           <t>RFQ</t>
         </is>
       </c>
-      <c r="E17" s="7" t="n">
+      <c r="F17" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="G17" s="9" t="n"/>
-      <c r="H17" s="10" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I17" s="9">
-        <f>IFERROR($E17*$G17,"")</f>
-        <v/>
-      </c>
-      <c r="J17" s="11" t="inlineStr">
+      <c r="H17" s="9" t="n"/>
+      <c r="I17" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J17" s="9">
+        <f>IFERROR($F17*$H17,"")</f>
+        <v/>
+      </c>
+      <c r="K17" s="11" t="inlineStr">
         <is>
           <t>6 × 80TE on the P&amp;ID</t>
         </is>
@@ -1428,23 +1446,23 @@
           <t>RULE</t>
         </is>
       </c>
-      <c r="E18" s="12" t="n">
+      <c r="F18" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="F18" s="12" t="inlineStr">
+      <c r="G18" s="12" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="G18" s="14" t="n"/>
-      <c r="H18" s="15" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I18" s="14">
-        <f>IFERROR($E18*$G18,"")</f>
-        <v/>
-      </c>
-      <c r="J18" s="16" t="inlineStr">
+      <c r="H18" s="14" t="n"/>
+      <c r="I18" s="15" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J18" s="14">
+        <f>IFERROR($F18*$H18,"")</f>
+        <v/>
+      </c>
+      <c r="K18" s="16" t="inlineStr">
         <is>
           <t>rule: 1 per 80TE connection</t>
         </is>
@@ -1467,23 +1485,23 @@
           <t>RULE</t>
         </is>
       </c>
-      <c r="E19" s="12" t="n">
+      <c r="F19" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="F19" s="12" t="inlineStr">
+      <c r="G19" s="12" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="G19" s="14" t="n"/>
-      <c r="H19" s="15" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I19" s="14">
-        <f>IFERROR($E19*$G19,"")</f>
-        <v/>
-      </c>
-      <c r="J19" s="16" t="inlineStr">
+      <c r="H19" s="14" t="n"/>
+      <c r="I19" s="15" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J19" s="14">
+        <f>IFERROR($F19*$H19,"")</f>
+        <v/>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
         <is>
           <t>rule: 1 per 80TE connection</t>
         </is>
@@ -1506,23 +1524,23 @@
           <t>RFQ</t>
         </is>
       </c>
-      <c r="E20" s="7" t="n">
+      <c r="F20" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="G20" s="9" t="n"/>
-      <c r="H20" s="10" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I20" s="9">
-        <f>IFERROR($E20*$G20,"")</f>
-        <v/>
-      </c>
-      <c r="J20" s="11" t="inlineStr">
+      <c r="H20" s="9" t="n"/>
+      <c r="I20" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J20" s="9">
+        <f>IFERROR($F20*$H20,"")</f>
+        <v/>
+      </c>
+      <c r="K20" s="11" t="inlineStr">
         <is>
           <t>2 × 40PN on the P&amp;ID</t>
         </is>
@@ -1545,23 +1563,23 @@
           <t>RULE</t>
         </is>
       </c>
-      <c r="E21" s="12" t="n">
+      <c r="F21" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="F21" s="12" t="inlineStr">
+      <c r="G21" s="12" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="G21" s="14" t="n"/>
-      <c r="H21" s="15" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I21" s="14">
-        <f>IFERROR($E21*$G21,"")</f>
-        <v/>
-      </c>
-      <c r="J21" s="16" t="inlineStr">
+      <c r="H21" s="14" t="n"/>
+      <c r="I21" s="15" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J21" s="14">
+        <f>IFERROR($F21*$H21,"")</f>
+        <v/>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
         <is>
           <t>rule: 1 per 40PN connection</t>
         </is>
@@ -1584,23 +1602,23 @@
           <t>RULE</t>
         </is>
       </c>
-      <c r="E22" s="12" t="n">
+      <c r="F22" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="F22" s="12" t="inlineStr">
+      <c r="G22" s="12" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="G22" s="14" t="n"/>
-      <c r="H22" s="15" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I22" s="14">
-        <f>IFERROR($E22*$G22,"")</f>
-        <v/>
-      </c>
-      <c r="J22" s="16" t="inlineStr">
+      <c r="H22" s="14" t="n"/>
+      <c r="I22" s="15" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J22" s="14">
+        <f>IFERROR($F22*$H22,"")</f>
+        <v/>
+      </c>
+      <c r="K22" s="16" t="inlineStr">
         <is>
           <t>rule: 1 per 40PN connection</t>
         </is>
@@ -1623,23 +1641,23 @@
           <t>RFQ</t>
         </is>
       </c>
-      <c r="E23" s="7" t="n">
+      <c r="F23" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="F23" s="7" t="inlineStr">
+      <c r="G23" s="7" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="G23" s="9" t="n"/>
-      <c r="H23" s="10" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I23" s="9">
-        <f>IFERROR($E23*$G23,"")</f>
-        <v/>
-      </c>
-      <c r="J23" s="11" t="inlineStr">
+      <c r="H23" s="9" t="n"/>
+      <c r="I23" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J23" s="9">
+        <f>IFERROR($F23*$H23,"")</f>
+        <v/>
+      </c>
+      <c r="K23" s="11" t="inlineStr">
         <is>
           <t>1 × 65PN on the P&amp;ID</t>
         </is>
@@ -1662,23 +1680,23 @@
           <t>RULE</t>
         </is>
       </c>
-      <c r="E24" s="12" t="n">
+      <c r="F24" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F24" s="12" t="inlineStr">
+      <c r="G24" s="12" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="G24" s="14" t="n"/>
-      <c r="H24" s="15" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I24" s="14">
-        <f>IFERROR($E24*$G24,"")</f>
-        <v/>
-      </c>
-      <c r="J24" s="16" t="inlineStr">
+      <c r="H24" s="14" t="n"/>
+      <c r="I24" s="15" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J24" s="14">
+        <f>IFERROR($F24*$H24,"")</f>
+        <v/>
+      </c>
+      <c r="K24" s="16" t="inlineStr">
         <is>
           <t>rule: 1 per 65PN connection</t>
         </is>
@@ -1701,23 +1719,23 @@
           <t>RULE</t>
         </is>
       </c>
-      <c r="E25" s="12" t="n">
+      <c r="F25" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F25" s="12" t="inlineStr">
+      <c r="G25" s="12" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="G25" s="14" t="n"/>
-      <c r="H25" s="15" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I25" s="14">
-        <f>IFERROR($E25*$G25,"")</f>
-        <v/>
-      </c>
-      <c r="J25" s="16" t="inlineStr">
+      <c r="H25" s="14" t="n"/>
+      <c r="I25" s="15" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J25" s="14">
+        <f>IFERROR($F25*$H25,"")</f>
+        <v/>
+      </c>
+      <c r="K25" s="16" t="inlineStr">
         <is>
           <t>rule: 1 per 65PN connection</t>
         </is>
@@ -1740,23 +1758,23 @@
           <t>RFQ</t>
         </is>
       </c>
-      <c r="E26" s="7" t="n">
+      <c r="F26" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="F26" s="7" t="inlineStr">
+      <c r="G26" s="7" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="G26" s="9" t="n"/>
-      <c r="H26" s="10" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I26" s="9">
-        <f>IFERROR($E26*$G26,"")</f>
-        <v/>
-      </c>
-      <c r="J26" s="11" t="inlineStr">
+      <c r="H26" s="9" t="n"/>
+      <c r="I26" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J26" s="9">
+        <f>IFERROR($F26*$H26,"")</f>
+        <v/>
+      </c>
+      <c r="K26" s="11" t="inlineStr">
         <is>
           <t>1 × 65TE on the P&amp;ID</t>
         </is>
@@ -1779,23 +1797,23 @@
           <t>RULE</t>
         </is>
       </c>
-      <c r="E27" s="12" t="n">
+      <c r="F27" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F27" s="12" t="inlineStr">
+      <c r="G27" s="12" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="G27" s="14" t="n"/>
-      <c r="H27" s="15" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I27" s="14">
-        <f>IFERROR($E27*$G27,"")</f>
-        <v/>
-      </c>
-      <c r="J27" s="16" t="inlineStr">
+      <c r="H27" s="14" t="n"/>
+      <c r="I27" s="15" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J27" s="14">
+        <f>IFERROR($F27*$H27,"")</f>
+        <v/>
+      </c>
+      <c r="K27" s="16" t="inlineStr">
         <is>
           <t>rule: 1 per 65TE connection</t>
         </is>
@@ -1818,23 +1836,23 @@
           <t>RULE</t>
         </is>
       </c>
-      <c r="E28" s="12" t="n">
+      <c r="F28" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F28" s="12" t="inlineStr">
+      <c r="G28" s="12" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="G28" s="14" t="n"/>
-      <c r="H28" s="15" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I28" s="14">
-        <f>IFERROR($E28*$G28,"")</f>
-        <v/>
-      </c>
-      <c r="J28" s="16" t="inlineStr">
+      <c r="H28" s="14" t="n"/>
+      <c r="I28" s="15" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J28" s="14">
+        <f>IFERROR($F28*$H28,"")</f>
+        <v/>
+      </c>
+      <c r="K28" s="16" t="inlineStr">
         <is>
           <t>rule: 1 per 65TE connection</t>
         </is>
@@ -1856,20 +1874,20 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="G29" s="5" t="n"/>
-      <c r="H29" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I29" s="5">
-        <f>IFERROR($E29*$G29,"")</f>
-        <v/>
-      </c>
-      <c r="J29" s="2" t="inlineStr">
+      <c r="H29" s="5" t="n"/>
+      <c r="I29" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J29" s="5">
+        <f>IFERROR($F29*$H29,"")</f>
+        <v/>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
         <is>
           <t>8 runs on the P&amp;ID</t>
         </is>
@@ -1891,20 +1909,20 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="G30" s="5" t="n"/>
-      <c r="H30" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I30" s="5">
-        <f>IFERROR($E30*$G30,"")</f>
-        <v/>
-      </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="H30" s="5" t="n"/>
+      <c r="I30" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J30" s="5">
+        <f>IFERROR($F30*$H30,"")</f>
+        <v/>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
         <is>
           <t>1 runs on the P&amp;ID</t>
         </is>
@@ -1926,20 +1944,20 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="G31" s="5" t="n"/>
-      <c r="H31" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I31" s="5">
-        <f>IFERROR($E31*$G31,"")</f>
-        <v/>
-      </c>
-      <c r="J31" s="2" t="inlineStr">
+      <c r="H31" s="5" t="n"/>
+      <c r="I31" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J31" s="5">
+        <f>IFERROR($F31*$H31,"")</f>
+        <v/>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>1 runs on the P&amp;ID</t>
         </is>
@@ -1961,20 +1979,20 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="G32" s="5" t="n"/>
-      <c r="H32" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I32" s="5">
-        <f>IFERROR($E32*$G32,"")</f>
-        <v/>
-      </c>
-      <c r="J32" s="2" t="inlineStr">
+      <c r="H32" s="5" t="n"/>
+      <c r="I32" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J32" s="5">
+        <f>IFERROR($F32*$H32,"")</f>
+        <v/>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
         <is>
           <t>1 runs on the P&amp;ID</t>
         </is>
@@ -1996,20 +2014,20 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="G33" s="5" t="n"/>
-      <c r="H33" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I33" s="5">
-        <f>IFERROR($E33*$G33,"")</f>
-        <v/>
-      </c>
-      <c r="J33" s="2" t="inlineStr">
+      <c r="H33" s="5" t="n"/>
+      <c r="I33" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J33" s="5">
+        <f>IFERROR($F33*$H33,"")</f>
+        <v/>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
         <is>
           <t>1 runs on the P&amp;ID</t>
         </is>
@@ -2031,20 +2049,20 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="G34" s="5" t="n"/>
-      <c r="H34" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I34" s="5">
-        <f>IFERROR($E34*$G34,"")</f>
-        <v/>
-      </c>
-      <c r="J34" s="2" t="inlineStr">
+      <c r="H34" s="5" t="n"/>
+      <c r="I34" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J34" s="5">
+        <f>IFERROR($F34*$H34,"")</f>
+        <v/>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>1 runs on the P&amp;ID</t>
         </is>
@@ -2066,20 +2084,20 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="G35" s="5" t="n"/>
-      <c r="H35" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I35" s="5">
-        <f>IFERROR($E35*$G35,"")</f>
-        <v/>
-      </c>
-      <c r="J35" s="2" t="inlineStr">
+      <c r="H35" s="5" t="n"/>
+      <c r="I35" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J35" s="5">
+        <f>IFERROR($F35*$H35,"")</f>
+        <v/>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>1 runs on the P&amp;ID</t>
         </is>
@@ -2102,21 +2120,21 @@
           <t>RATE</t>
         </is>
       </c>
-      <c r="E36" s="12" t="n"/>
-      <c r="F36" s="12" t="inlineStr">
+      <c r="F36" s="12" t="n"/>
+      <c r="G36" s="12" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="G36" s="14" t="n"/>
-      <c r="H36" s="15" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I36" s="14">
-        <f>IFERROR($E36*$G36,"")</f>
-        <v/>
-      </c>
-      <c r="J36" s="16" t="inlineStr">
+      <c r="H36" s="14" t="n"/>
+      <c r="I36" s="15" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J36" s="14">
+        <f>IFERROR($F36*$H36,"")</f>
+        <v/>
+      </c>
+      <c r="K36" s="16" t="inlineStr">
         <is>
           <t>rate card by diameter</t>
         </is>
@@ -2138,20 +2156,20 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>lot</t>
         </is>
       </c>
-      <c r="G37" s="5" t="n"/>
-      <c r="H37" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I37" s="5">
-        <f>IFERROR($E37*$G37,"")</f>
-        <v/>
-      </c>
-      <c r="J37" s="2" t="inlineStr">
+      <c r="H37" s="5" t="n"/>
+      <c r="I37" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J37" s="5">
+        <f>IFERROR($F37*$H37,"")</f>
+        <v/>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
         <is>
           <t>carried on past jobs</t>
         </is>
@@ -2176,6 +2194,7 @@
       <c r="H38" s="6" t="n"/>
       <c r="I38" s="6" t="n"/>
       <c r="J38" s="6" t="n"/>
+      <c r="K38" s="6" t="n"/>
     </row>
     <row r="39">
       <c r="B39" s="17" t="inlineStr">
@@ -2193,22 +2212,27 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="E39" s="19" t="inlineStr">
+        <is>
+          <t>In-house</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
         <is>
           <t>hr</t>
         </is>
       </c>
-      <c r="G39" s="5" t="n">
+      <c r="H39" s="5" t="n">
         <v>105</v>
       </c>
-      <c r="H39" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I39" s="5">
-        <f>IFERROR($E39*$G39,"")</f>
-        <v/>
-      </c>
-      <c r="J39" s="2" t="inlineStr">
+      <c r="I39" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J39" s="5">
+        <f>IFERROR($F39*$H39,"")</f>
+        <v/>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
         <is>
           <t>crew × days</t>
         </is>
@@ -2230,22 +2254,27 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="E40" s="19" t="inlineStr">
+        <is>
+          <t>In-house</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
         <is>
           <t>hr</t>
         </is>
       </c>
-      <c r="G40" s="5" t="n">
+      <c r="H40" s="5" t="n">
         <v>105</v>
       </c>
-      <c r="H40" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I40" s="5">
-        <f>IFERROR($E40*$G40,"")</f>
-        <v/>
-      </c>
-      <c r="J40" s="2" t="inlineStr">
+      <c r="I40" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J40" s="5">
+        <f>IFERROR($F40*$H40,"")</f>
+        <v/>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
         <is>
           <t>crew × days</t>
         </is>
@@ -2267,22 +2296,27 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="E41" s="19" t="inlineStr">
+        <is>
+          <t>In-house</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
         <is>
           <t>hr</t>
         </is>
       </c>
-      <c r="G41" s="5" t="n">
+      <c r="H41" s="5" t="n">
         <v>105</v>
       </c>
-      <c r="H41" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I41" s="5">
-        <f>IFERROR($E41*$G41,"")</f>
-        <v/>
-      </c>
-      <c r="J41" s="2" t="inlineStr">
+      <c r="I41" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J41" s="5">
+        <f>IFERROR($F41*$H41,"")</f>
+        <v/>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
         <is>
           <t>crew × days</t>
         </is>
@@ -2304,22 +2338,27 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="E42" s="19" t="inlineStr">
+        <is>
+          <t>In-house</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
         <is>
           <t>hr</t>
         </is>
       </c>
-      <c r="G42" s="5" t="n">
+      <c r="H42" s="5" t="n">
         <v>105</v>
       </c>
-      <c r="H42" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I42" s="5">
-        <f>IFERROR($E42*$G42,"")</f>
-        <v/>
-      </c>
-      <c r="J42" s="2" t="inlineStr">
+      <c r="I42" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J42" s="5">
+        <f>IFERROR($F42*$H42,"")</f>
+        <v/>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
         <is>
           <t>crew × days</t>
         </is>
@@ -2341,22 +2380,27 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="E43" s="19" t="inlineStr">
+        <is>
+          <t>In-house</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
         <is>
           <t>hr</t>
         </is>
       </c>
-      <c r="G43" s="5" t="n">
+      <c r="H43" s="5" t="n">
         <v>105</v>
       </c>
-      <c r="H43" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I43" s="5">
-        <f>IFERROR($E43*$G43,"")</f>
-        <v/>
-      </c>
-      <c r="J43" s="2" t="inlineStr">
+      <c r="I43" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J43" s="5">
+        <f>IFERROR($F43*$H43,"")</f>
+        <v/>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
         <is>
           <t>crew × days</t>
         </is>
@@ -2378,22 +2422,27 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="E44" s="19" t="inlineStr">
+        <is>
+          <t>In-house</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
         <is>
           <t>hr</t>
         </is>
       </c>
-      <c r="G44" s="5" t="n">
+      <c r="H44" s="5" t="n">
         <v>105</v>
       </c>
-      <c r="H44" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I44" s="5">
-        <f>IFERROR($E44*$G44,"")</f>
-        <v/>
-      </c>
-      <c r="J44" s="2" t="inlineStr">
+      <c r="I44" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J44" s="5">
+        <f>IFERROR($F44*$H44,"")</f>
+        <v/>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
         <is>
           <t>crew × days</t>
         </is>
@@ -2415,22 +2464,27 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="E45" s="19" t="inlineStr">
+        <is>
+          <t>In-house</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
         <is>
           <t>hr</t>
         </is>
       </c>
-      <c r="G45" s="5" t="n">
+      <c r="H45" s="5" t="n">
         <v>105</v>
       </c>
-      <c r="H45" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I45" s="5">
-        <f>IFERROR($E45*$G45,"")</f>
-        <v/>
-      </c>
-      <c r="J45" s="2" t="inlineStr">
+      <c r="I45" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J45" s="5">
+        <f>IFERROR($F45*$H45,"")</f>
+        <v/>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
         <is>
           <t>crew × days</t>
         </is>
@@ -2452,22 +2506,27 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="E46" s="19" t="inlineStr">
+        <is>
+          <t>In-house</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
         <is>
           <t>hr</t>
         </is>
       </c>
-      <c r="G46" s="5" t="n">
+      <c r="H46" s="5" t="n">
         <v>105</v>
       </c>
-      <c r="H46" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I46" s="5">
-        <f>IFERROR($E46*$G46,"")</f>
-        <v/>
-      </c>
-      <c r="J46" s="2" t="inlineStr">
+      <c r="I46" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J46" s="5">
+        <f>IFERROR($F46*$H46,"")</f>
+        <v/>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
         <is>
           <t>crew × days</t>
         </is>
@@ -2489,22 +2548,27 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="E47" s="19" t="inlineStr">
+        <is>
+          <t>In-house</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
         <is>
           <t>hr</t>
         </is>
       </c>
-      <c r="G47" s="5" t="n">
+      <c r="H47" s="5" t="n">
         <v>105</v>
       </c>
-      <c r="H47" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I47" s="5">
-        <f>IFERROR($E47*$G47,"")</f>
-        <v/>
-      </c>
-      <c r="J47" s="2" t="inlineStr">
+      <c r="I47" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J47" s="5">
+        <f>IFERROR($F47*$H47,"")</f>
+        <v/>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
         <is>
           <t>crew × days</t>
         </is>
@@ -2526,20 +2590,20 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="G48" t="inlineStr">
         <is>
           <t>lot</t>
         </is>
       </c>
-      <c r="G48" s="5" t="n"/>
-      <c r="H48" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I48" s="5">
-        <f>IFERROR($E48*$G48,"")</f>
-        <v/>
-      </c>
-      <c r="J48" s="2" t="inlineStr">
+      <c r="H48" s="5" t="n"/>
+      <c r="I48" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J48" s="5">
+        <f>IFERROR($F48*$H48,"")</f>
+        <v/>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
         <is>
           <t>carried on past jobs</t>
         </is>
@@ -2561,20 +2625,20 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="G49" t="inlineStr">
         <is>
           <t>lot</t>
         </is>
       </c>
-      <c r="G49" s="5" t="n"/>
-      <c r="H49" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I49" s="5">
-        <f>IFERROR($E49*$G49,"")</f>
-        <v/>
-      </c>
-      <c r="J49" s="2" t="inlineStr">
+      <c r="H49" s="5" t="n"/>
+      <c r="I49" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J49" s="5">
+        <f>IFERROR($F49*$H49,"")</f>
+        <v/>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
         <is>
           <t>carried on past jobs</t>
         </is>
@@ -2596,20 +2660,20 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="G50" t="inlineStr">
         <is>
           <t>lot</t>
         </is>
       </c>
-      <c r="G50" s="5" t="n"/>
-      <c r="H50" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I50" s="5">
-        <f>IFERROR($E50*$G50,"")</f>
-        <v/>
-      </c>
-      <c r="J50" s="2" t="inlineStr">
+      <c r="H50" s="5" t="n"/>
+      <c r="I50" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J50" s="5">
+        <f>IFERROR($F50*$H50,"")</f>
+        <v/>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
         <is>
           <t>carried on past jobs</t>
         </is>
@@ -2634,6 +2698,7 @@
       <c r="H51" s="6" t="n"/>
       <c r="I51" s="6" t="n"/>
       <c r="J51" s="6" t="n"/>
+      <c r="K51" s="6" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="n"/>
@@ -2652,23 +2717,28 @@
           <t>RFQ</t>
         </is>
       </c>
-      <c r="E52" s="7" t="n">
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>Subcontract</t>
+        </is>
+      </c>
+      <c r="F52" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="F52" s="7" t="inlineStr">
+      <c r="G52" s="7" t="inlineStr">
         <is>
           <t>lot</t>
         </is>
       </c>
-      <c r="G52" s="9" t="n"/>
-      <c r="H52" s="10" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I52" s="9">
-        <f>IFERROR($E52*$G52,"")</f>
-        <v/>
-      </c>
-      <c r="J52" s="11" t="inlineStr">
+      <c r="H52" s="9" t="n"/>
+      <c r="I52" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J52" s="9">
+        <f>IFERROR($F52*$H52,"")</f>
+        <v/>
+      </c>
+      <c r="K52" s="11" t="inlineStr">
         <is>
           <t>from the maximum demand schedule</t>
         </is>
@@ -2691,23 +2761,28 @@
           <t>RFQ</t>
         </is>
       </c>
-      <c r="E53" s="7" t="n">
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>Subcontract</t>
+        </is>
+      </c>
+      <c r="F53" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="F53" s="7" t="inlineStr">
+      <c r="G53" s="7" t="inlineStr">
         <is>
           <t>lot</t>
         </is>
       </c>
-      <c r="G53" s="9" t="n"/>
-      <c r="H53" s="10" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I53" s="9">
-        <f>IFERROR($E53*$G53,"")</f>
-        <v/>
-      </c>
-      <c r="J53" s="11" t="inlineStr">
+      <c r="H53" s="9" t="n"/>
+      <c r="I53" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J53" s="9">
+        <f>IFERROR($F53*$H53,"")</f>
+        <v/>
+      </c>
+      <c r="K53" s="11" t="inlineStr">
         <is>
           <t>electrical contractor</t>
         </is>
@@ -2732,6 +2807,7 @@
       <c r="H54" s="6" t="n"/>
       <c r="I54" s="6" t="n"/>
       <c r="J54" s="6" t="n"/>
+      <c r="K54" s="6" t="n"/>
     </row>
     <row r="55">
       <c r="B55" s="17" t="inlineStr">
@@ -2749,22 +2825,27 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
+      <c r="E55" s="19" t="inlineStr">
+        <is>
+          <t>In-house</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
         <is>
           <t>hr</t>
         </is>
       </c>
-      <c r="G55" s="5" t="n">
+      <c r="H55" s="5" t="n">
         <v>140</v>
       </c>
-      <c r="H55" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I55" s="5">
-        <f>IFERROR($E55*$G55,"")</f>
-        <v/>
-      </c>
-      <c r="J55" s="2" t="inlineStr">
+      <c r="I55" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J55" s="5">
+        <f>IFERROR($F55*$H55,"")</f>
+        <v/>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
         <is>
           <t>hours to be entered</t>
         </is>
@@ -2786,22 +2867,27 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="E56" s="19" t="inlineStr">
+        <is>
+          <t>In-house</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
         <is>
           <t>hr</t>
         </is>
       </c>
-      <c r="G56" s="5" t="n">
+      <c r="H56" s="5" t="n">
         <v>140</v>
       </c>
-      <c r="H56" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I56" s="5">
-        <f>IFERROR($E56*$G56,"")</f>
-        <v/>
-      </c>
-      <c r="J56" s="2" t="inlineStr">
+      <c r="I56" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J56" s="5">
+        <f>IFERROR($F56*$H56,"")</f>
+        <v/>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
         <is>
           <t>hours to be entered</t>
         </is>
@@ -2823,22 +2909,27 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
+      <c r="E57" s="19" t="inlineStr">
+        <is>
+          <t>In-house</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
         <is>
           <t>hr</t>
         </is>
       </c>
-      <c r="G57" s="5" t="n">
+      <c r="H57" s="5" t="n">
         <v>140</v>
       </c>
-      <c r="H57" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I57" s="5">
-        <f>IFERROR($E57*$G57,"")</f>
-        <v/>
-      </c>
-      <c r="J57" s="2" t="inlineStr">
+      <c r="I57" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J57" s="5">
+        <f>IFERROR($F57*$H57,"")</f>
+        <v/>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
         <is>
           <t>hours to be entered</t>
         </is>
@@ -2860,22 +2951,27 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="E58" s="19" t="inlineStr">
+        <is>
+          <t>In-house</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
         <is>
           <t>hr</t>
         </is>
       </c>
-      <c r="G58" s="5" t="n">
+      <c r="H58" s="5" t="n">
         <v>140</v>
       </c>
-      <c r="H58" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I58" s="5">
-        <f>IFERROR($E58*$G58,"")</f>
-        <v/>
-      </c>
-      <c r="J58" s="2" t="inlineStr">
+      <c r="I58" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J58" s="5">
+        <f>IFERROR($F58*$H58,"")</f>
+        <v/>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
         <is>
           <t>hours to be entered</t>
         </is>
@@ -2897,20 +2993,20 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr">
+      <c r="G59" t="inlineStr">
         <is>
           <t>lot</t>
         </is>
       </c>
-      <c r="G59" s="5" t="n"/>
-      <c r="H59" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I59" s="5">
-        <f>IFERROR($E59*$G59,"")</f>
-        <v/>
-      </c>
-      <c r="J59" s="2" t="inlineStr">
+      <c r="H59" s="5" t="n"/>
+      <c r="I59" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J59" s="5">
+        <f>IFERROR($F59*$H59,"")</f>
+        <v/>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
         <is>
           <t>carried on past jobs</t>
         </is>
@@ -2935,6 +3031,7 @@
       <c r="H60" s="6" t="n"/>
       <c r="I60" s="6" t="n"/>
       <c r="J60" s="6" t="n"/>
+      <c r="K60" s="6" t="n"/>
     </row>
     <row r="61">
       <c r="B61" s="17" t="inlineStr">
@@ -2952,22 +3049,27 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
+      <c r="E61" s="19" t="inlineStr">
+        <is>
+          <t>In-house</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
         <is>
           <t>hr</t>
         </is>
       </c>
-      <c r="G61" s="5" t="n">
+      <c r="H61" s="5" t="n">
         <v>105</v>
       </c>
-      <c r="H61" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I61" s="5">
-        <f>IFERROR($E61*$G61,"")</f>
-        <v/>
-      </c>
-      <c r="J61" s="2" t="inlineStr">
+      <c r="I61" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J61" s="5">
+        <f>IFERROR($F61*$H61,"")</f>
+        <v/>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
         <is>
           <t>to be entered</t>
         </is>
@@ -2989,20 +3091,20 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
+      <c r="G62" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G62" s="5" t="n"/>
-      <c r="H62" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I62" s="5">
-        <f>IFERROR($E62*$G62,"")</f>
-        <v/>
-      </c>
-      <c r="J62" s="2" t="inlineStr">
+      <c r="H62" s="5" t="n"/>
+      <c r="I62" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J62" s="5">
+        <f>IFERROR($F62*$H62,"")</f>
+        <v/>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
         <is>
           <t>to be entered</t>
         </is>
@@ -3024,20 +3126,20 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="G63" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="G63" s="5" t="n"/>
-      <c r="H63" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I63" s="5">
-        <f>IFERROR($E63*$G63,"")</f>
-        <v/>
-      </c>
-      <c r="J63" s="2" t="inlineStr">
+      <c r="H63" s="5" t="n"/>
+      <c r="I63" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J63" s="5">
+        <f>IFERROR($F63*$H63,"")</f>
+        <v/>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
         <is>
           <t>to be entered</t>
         </is>
@@ -3062,6 +3164,7 @@
       <c r="H64" s="6" t="n"/>
       <c r="I64" s="6" t="n"/>
       <c r="J64" s="6" t="n"/>
+      <c r="K64" s="6" t="n"/>
     </row>
     <row r="65">
       <c r="B65" s="17" t="inlineStr">
@@ -3079,23 +3182,23 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="E65" t="n">
+      <c r="F65" t="n">
         <v>4</v>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="G65" t="inlineStr">
         <is>
           <t>visit</t>
         </is>
       </c>
-      <c r="G65" s="5" t="n"/>
-      <c r="H65" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I65" s="5">
-        <f>IFERROR($E65*$G65,"")</f>
-        <v/>
-      </c>
-      <c r="J65" s="2" t="inlineStr">
+      <c r="H65" s="5" t="n"/>
+      <c r="I65" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J65" s="5">
+        <f>IFERROR($F65*$H65,"")</f>
+        <v/>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
         <is>
           <t>rate to be entered</t>
         </is>
@@ -3117,26 +3220,31 @@
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr">
+      <c r="G66" t="inlineStr">
         <is>
           <t>lot</t>
         </is>
       </c>
-      <c r="G66" s="5" t="n"/>
-      <c r="H66" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I66" s="5">
-        <f>IFERROR($E66*$G66,"")</f>
-        <v/>
-      </c>
-      <c r="J66" s="2" t="inlineStr">
+      <c r="H66" s="5" t="n"/>
+      <c r="I66" s="18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J66" s="5">
+        <f>IFERROR($F66*$H66,"")</f>
+        <v/>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
         <is>
           <t>carried on past jobs</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="E39 E40 E41 E42 E43 E44 E45 E46 E47 E52 E53 E55 E56 E57 E58 E61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"In-house,Subcontract"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3801,11 +3909,11 @@
       <c r="D2" t="n">
         <v>10</v>
       </c>
-      <c r="E2" s="19">
+      <c r="E2" s="20">
         <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B2,'Welding hours'!$C$3:$C$14,0),MATCH($C2,'Welding hours'!$D$2:$O$2,0)),0)</f>
         <v/>
       </c>
-      <c r="F2" s="19">
+      <c r="F2" s="20">
         <f>D2*E2</f>
         <v/>
       </c>
@@ -3834,11 +3942,11 @@
       <c r="D3" t="n">
         <v>0</v>
       </c>
-      <c r="E3" s="19">
+      <c r="E3" s="20">
         <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B3,'Welding hours'!$C$3:$C$14,0),MATCH($C3,'Welding hours'!$D$2:$O$2,0)),0)</f>
         <v/>
       </c>
-      <c r="F3" s="19">
+      <c r="F3" s="20">
         <f>D3*E3</f>
         <v/>
       </c>
@@ -3867,11 +3975,11 @@
       <c r="D4" t="n">
         <v>6</v>
       </c>
-      <c r="E4" s="19">
+      <c r="E4" s="20">
         <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B4,'Welding hours'!$C$3:$C$14,0),MATCH($C4,'Welding hours'!$D$2:$O$2,0)),0)</f>
         <v/>
       </c>
-      <c r="F4" s="19">
+      <c r="F4" s="20">
         <f>D4*E4</f>
         <v/>
       </c>
@@ -3900,11 +4008,11 @@
       <c r="D5" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="19">
+      <c r="E5" s="20">
         <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B5,'Welding hours'!$C$3:$C$14,0),MATCH($C5,'Welding hours'!$D$2:$O$2,0)),0)</f>
         <v/>
       </c>
-      <c r="F5" s="19">
+      <c r="F5" s="20">
         <f>D5*E5</f>
         <v/>
       </c>
@@ -3933,11 +4041,11 @@
       <c r="D6" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="19">
+      <c r="E6" s="20">
         <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B6,'Welding hours'!$C$3:$C$14,0),MATCH($C6,'Welding hours'!$D$2:$O$2,0)),0)</f>
         <v/>
       </c>
-      <c r="F6" s="19">
+      <c r="F6" s="20">
         <f>D6*E6</f>
         <v/>
       </c>
@@ -3966,11 +4074,11 @@
       <c r="D7" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="19">
+      <c r="E7" s="20">
         <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B7,'Welding hours'!$C$3:$C$14,0),MATCH($C7,'Welding hours'!$D$2:$O$2,0)),0)</f>
         <v/>
       </c>
-      <c r="F7" s="19">
+      <c r="F7" s="20">
         <f>D7*E7</f>
         <v/>
       </c>
@@ -3999,11 +4107,11 @@
       <c r="D8" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="19">
+      <c r="E8" s="20">
         <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B8,'Welding hours'!$C$3:$C$14,0),MATCH($C8,'Welding hours'!$D$2:$O$2,0)),0)</f>
         <v/>
       </c>
-      <c r="F8" s="19">
+      <c r="F8" s="20">
         <f>D8*E8</f>
         <v/>
       </c>
@@ -4032,11 +4140,11 @@
       <c r="D9" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="19">
+      <c r="E9" s="20">
         <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B9,'Welding hours'!$C$3:$C$14,0),MATCH($C9,'Welding hours'!$D$2:$O$2,0)),0)</f>
         <v/>
       </c>
-      <c r="F9" s="19">
+      <c r="F9" s="20">
         <f>D9*E9</f>
         <v/>
       </c>
@@ -4065,11 +4173,11 @@
       <c r="D10" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="19">
+      <c r="E10" s="20">
         <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B10,'Welding hours'!$C$3:$C$14,0),MATCH($C10,'Welding hours'!$D$2:$O$2,0)),0)</f>
         <v/>
       </c>
-      <c r="F10" s="19">
+      <c r="F10" s="20">
         <f>D10*E10</f>
         <v/>
       </c>
@@ -4098,11 +4206,11 @@
       <c r="D11" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="19">
+      <c r="E11" s="20">
         <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B11,'Welding hours'!$C$3:$C$14,0),MATCH($C11,'Welding hours'!$D$2:$O$2,0)),0)</f>
         <v/>
       </c>
-      <c r="F11" s="19">
+      <c r="F11" s="20">
         <f>D11*E11</f>
         <v/>
       </c>
@@ -4129,11 +4237,11 @@
         </is>
       </c>
       <c r="D12" s="12" t="n"/>
-      <c r="E12" s="20">
+      <c r="E12" s="21">
         <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B12,'Welding hours'!$C$3:$C$14,0),MATCH($C12,'Welding hours'!$D$2:$O$2,0)),0)</f>
         <v/>
       </c>
-      <c r="F12" s="20">
+      <c r="F12" s="21">
         <f>D12*E12</f>
         <v/>
       </c>
@@ -4160,11 +4268,11 @@
         </is>
       </c>
       <c r="D13" s="12" t="n"/>
-      <c r="E13" s="20">
+      <c r="E13" s="21">
         <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B13,'Welding hours'!$C$3:$C$14,0),MATCH($C13,'Welding hours'!$D$2:$O$2,0)),0)</f>
         <v/>
       </c>
-      <c r="F13" s="20">
+      <c r="F13" s="21">
         <f>D13*E13</f>
         <v/>
       </c>
@@ -4191,11 +4299,11 @@
         </is>
       </c>
       <c r="D14" s="12" t="n"/>
-      <c r="E14" s="20">
+      <c r="E14" s="21">
         <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B14,'Welding hours'!$C$3:$C$14,0),MATCH($C14,'Welding hours'!$D$2:$O$2,0)),0)</f>
         <v/>
       </c>
-      <c r="F14" s="20">
+      <c r="F14" s="21">
         <f>D14*E14</f>
         <v/>
       </c>
@@ -4222,11 +4330,11 @@
         </is>
       </c>
       <c r="D15" s="12" t="n"/>
-      <c r="E15" s="20">
+      <c r="E15" s="21">
         <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B15,'Welding hours'!$C$3:$C$14,0),MATCH($C15,'Welding hours'!$D$2:$O$2,0)),0)</f>
         <v/>
       </c>
-      <c r="F15" s="20">
+      <c r="F15" s="21">
         <f>D15*E15</f>
         <v/>
       </c>
@@ -4253,11 +4361,11 @@
         </is>
       </c>
       <c r="D16" s="12" t="n"/>
-      <c r="E16" s="20">
+      <c r="E16" s="21">
         <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B16,'Welding hours'!$C$3:$C$14,0),MATCH($C16,'Welding hours'!$D$2:$O$2,0)),0)</f>
         <v/>
       </c>
-      <c r="F16" s="20">
+      <c r="F16" s="21">
         <f>D16*E16</f>
         <v/>
       </c>
@@ -4284,11 +4392,11 @@
         </is>
       </c>
       <c r="D17" s="12" t="n"/>
-      <c r="E17" s="20">
+      <c r="E17" s="21">
         <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B17,'Welding hours'!$C$3:$C$14,0),MATCH($C17,'Welding hours'!$D$2:$O$2,0)),0)</f>
         <v/>
       </c>
-      <c r="F17" s="20">
+      <c r="F17" s="21">
         <f>D17*E17</f>
         <v/>
       </c>
@@ -4315,11 +4423,11 @@
         </is>
       </c>
       <c r="D18" s="12" t="n"/>
-      <c r="E18" s="20">
+      <c r="E18" s="21">
         <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B18,'Welding hours'!$C$3:$C$14,0),MATCH($C18,'Welding hours'!$D$2:$O$2,0)),0)</f>
         <v/>
       </c>
-      <c r="F18" s="20">
+      <c r="F18" s="21">
         <f>D18*E18</f>
         <v/>
       </c>
@@ -4339,7 +4447,7 @@
       <c r="C20" s="3" t="n"/>
       <c r="D20" s="3" t="n"/>
       <c r="E20" s="3" t="n"/>
-      <c r="F20" s="21">
+      <c r="F20" s="22">
         <f>SUM(F2:F18)</f>
         <v/>
       </c>
@@ -4377,67 +4485,67 @@
   </cols>
   <sheetData>
     <row r="2">
-      <c r="C2" s="22" t="inlineStr">
+      <c r="C2" s="23" t="inlineStr">
         <is>
           <t>Rates</t>
         </is>
       </c>
-      <c r="D2" s="22" t="inlineStr">
+      <c r="D2" s="23" t="inlineStr">
         <is>
           <t>Weld Neck</t>
         </is>
       </c>
-      <c r="E2" s="22" t="inlineStr">
+      <c r="E2" s="23" t="inlineStr">
         <is>
           <t>Slip On</t>
         </is>
       </c>
-      <c r="F2" s="22" t="inlineStr">
+      <c r="F2" s="23" t="inlineStr">
         <is>
           <t>Blind</t>
         </is>
       </c>
-      <c r="G2" s="22" t="inlineStr">
+      <c r="G2" s="23" t="inlineStr">
         <is>
           <t>Socket Weld</t>
         </is>
       </c>
-      <c r="H2" s="22" t="inlineStr">
+      <c r="H2" s="23" t="inlineStr">
         <is>
           <t>Straight</t>
         </is>
       </c>
-      <c r="I2" s="22" t="inlineStr">
+      <c r="I2" s="23" t="inlineStr">
         <is>
           <t>Buttweld</t>
         </is>
       </c>
-      <c r="J2" s="22" t="inlineStr">
+      <c r="J2" s="23" t="inlineStr">
         <is>
           <t>Elbow</t>
         </is>
       </c>
-      <c r="K2" s="22" t="inlineStr">
+      <c r="K2" s="23" t="inlineStr">
         <is>
           <t>Tee</t>
         </is>
       </c>
-      <c r="L2" s="22" t="inlineStr">
+      <c r="L2" s="23" t="inlineStr">
         <is>
           <t>Reducer</t>
         </is>
       </c>
-      <c r="M2" s="22" t="inlineStr">
+      <c r="M2" s="23" t="inlineStr">
         <is>
           <t>Cap</t>
         </is>
       </c>
-      <c r="N2" s="22" t="inlineStr">
+      <c r="N2" s="23" t="inlineStr">
         <is>
           <t>Branch</t>
         </is>
       </c>
-      <c r="O2" s="22" t="inlineStr">
+      <c r="O2" s="23" t="inlineStr">
         <is>
           <t>Stab In</t>
         </is>
@@ -4977,7 +5085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5175,32 +5283,49 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>VSD / IE5 VSD / EC Fan Supply</t>
+          <t>in-house vs subcontract</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1 comms point</t>
+          <t>the code changes with it: L- own labour ↔ S- subcontract, E- own electrical ↔ ES- electrical sub</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>observed on past jobs</t>
+          <t>their own code families</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>VSD / IE5 VSD / EC Fan Supply</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1 comms point</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>observed on past jobs</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Motor Starter DOL</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>1 DI + 1 DO + 1 AO</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>observed on past jobs</t>
         </is>

</xml_diff>

<commit_message>
job-specific RFQs, live tender schedule, welding line
</commit_message>
<xml_diff>
--- a/quote-builder/Riverbend-Q900142-Costing.xlsx
+++ b/quote-builder/Riverbend-Q900142-Costing.xlsx
@@ -120,13 +120,13 @@
     <xf numFmtId="4" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -515,21 +515,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Riverbend Produce Limited</t>
+          <t>Riverbend Produce — Coolstore 3 Glycol Chilling Upgrade</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Coolstore 3 — Glycol Chilling Upgrade</t>
+          <t>Q900142</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Q900142 · Rev A</t>
+          <t>Rev A</t>
         </is>
       </c>
     </row>
@@ -813,766 +813,772 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n"/>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>50TE isolating valve</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>M-VG</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>BF-50TE</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>Bought in</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>PRICE LIST</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I4" s="16" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="J4" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K4" s="4">
+        <f>IFERROR($G4*$I4,"")</f>
+        <v/>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>10 × 50TE on the P&amp;ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>80TE isolating valve</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>M-VG</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>BF-80TE</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Bought in</t>
+        </is>
+      </c>
+      <c r="F5" s="15" t="inlineStr">
+        <is>
+          <t>PRICE LIST</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>6</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I5" s="16" t="n">
+        <v>112</v>
+      </c>
+      <c r="J5" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K5" s="4">
+        <f>IFERROR($G5*$I5,"")</f>
+        <v/>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>6 × 80TE on the P&amp;ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>40PN isolating valve</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>M-VG</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>BF-40PN</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>Bought in</t>
+        </is>
+      </c>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>PRICE LIST</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I6" s="16" t="n">
+        <v>121</v>
+      </c>
+      <c r="J6" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K6" s="4">
+        <f>IFERROR($G6*$I6,"")</f>
+        <v/>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>2 × 40PN on the P&amp;ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>65PN isolating valve</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>M-VG</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>BF-65PN</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>Bought in</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>PRICE LIST</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="n">
+        <v>168</v>
+      </c>
+      <c r="J7" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K7" s="4">
+        <f>IFERROR($G7*$I7,"")</f>
+        <v/>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>1 × 65PN on the P&amp;ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>65TE isolating valve</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>M-VG</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>BF-65TE</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>Bought in</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>PRICE LIST</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I8" s="16" t="n">
+        <v>138</v>
+      </c>
+      <c r="J8" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K8" s="4">
+        <f>IFERROR($G8*$I8,"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>1 × 65TE on the P&amp;ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n"/>
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Section 7.1 total</t>
         </is>
       </c>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="14">
-        <f>SUM(K3:K3)</f>
-        <v/>
-      </c>
-      <c r="L4" s="3" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="C9" s="3" t="n"/>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="n"/>
+      <c r="K9" s="18">
+        <f>SUM(K3:K8)</f>
+        <v/>
+      </c>
+      <c r="L9" s="3" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>7.2</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Evaporative condenser</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
-      <c r="E5" s="7" t="n"/>
-      <c r="F5" s="7" t="n"/>
-      <c r="G5" s="7" t="n"/>
-      <c r="H5" s="7" t="n"/>
-      <c r="I5" s="7" t="n"/>
-      <c r="J5" s="7" t="n"/>
-      <c r="K5" s="7" t="n"/>
-      <c r="L5" s="7" t="n"/>
-    </row>
-    <row r="6">
-      <c r="B6" s="8" t="inlineStr">
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7" t="n"/>
+      <c r="I10" s="7" t="n"/>
+      <c r="J10" s="7" t="n"/>
+      <c r="K10" s="7" t="n"/>
+      <c r="L10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Condenser</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>C-CON</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr"/>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr"/>
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>RFQ</t>
         </is>
       </c>
-      <c r="G6" s="9" t="n">
+      <c r="G11" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H6" s="9" t="inlineStr">
+      <c r="H11" s="9" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="I6" s="11" t="n"/>
-      <c r="J6" s="12" t="n">
+      <c r="I11" s="11" t="n"/>
+      <c r="J11" s="12" t="n">
         <v>0.15</v>
       </c>
-      <c r="K6" s="11">
-        <f>IFERROR($G6*$I6,"")</f>
-        <v/>
-      </c>
-      <c r="L6" s="13" t="inlineStr">
+      <c r="K11" s="11">
+        <f>IFERROR($G11*$I11,"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="13" t="inlineStr">
         <is>
           <t>620 kWR each · EC Fan Supply</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="n"/>
-      <c r="B7" s="3" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Section 7.2 total</t>
         </is>
       </c>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
-      <c r="F7" s="3" t="n"/>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
-      <c r="J7" s="3" t="n"/>
-      <c r="K7" s="14">
-        <f>SUM(K6:K6)</f>
-        <v/>
-      </c>
-      <c r="L7" s="3" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="3" t="n"/>
+      <c r="G12" s="3" t="n"/>
+      <c r="H12" s="3" t="n"/>
+      <c r="I12" s="3" t="n"/>
+      <c r="J12" s="3" t="n"/>
+      <c r="K12" s="18">
+        <f>SUM(K11:K11)</f>
+        <v/>
+      </c>
+      <c r="L12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>7.3</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Chiller plate heat exchanger</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="7" t="n"/>
-      <c r="H8" s="7" t="n"/>
-      <c r="I8" s="7" t="n"/>
-      <c r="J8" s="7" t="n"/>
-      <c r="K8" s="7" t="n"/>
-      <c r="L8" s="7" t="n"/>
-    </row>
-    <row r="9">
-      <c r="B9" s="8" t="inlineStr">
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
+      <c r="I13" s="7" t="n"/>
+      <c r="J13" s="7" t="n"/>
+      <c r="K13" s="7" t="n"/>
+      <c r="L13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Chiller Phe</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>C-HX</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr"/>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr"/>
+      <c r="E14" s="10" t="inlineStr">
         <is>
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>RFQ</t>
         </is>
       </c>
-      <c r="G9" s="9" t="n">
+      <c r="G14" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="9" t="inlineStr">
+      <c r="H14" s="9" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="I9" s="11" t="n"/>
-      <c r="J9" s="12" t="n">
+      <c r="I14" s="11" t="n"/>
+      <c r="J14" s="12" t="n">
         <v>0.15</v>
       </c>
-      <c r="K9" s="11">
-        <f>IFERROR($G9*$I9,"")</f>
-        <v/>
-      </c>
-      <c r="L9" s="13" t="inlineStr">
+      <c r="K14" s="11">
+        <f>IFERROR($G14*$I14,"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="13" t="inlineStr">
         <is>
           <t>520 kWR each · no starter shown</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="n"/>
-      <c r="B10" s="3" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Section 7.3 total</t>
         </is>
       </c>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="n"/>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
-      <c r="I10" s="3" t="n"/>
-      <c r="J10" s="3" t="n"/>
-      <c r="K10" s="14">
-        <f>SUM(K9:K9)</f>
-        <v/>
-      </c>
-      <c r="L10" s="3" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="3" t="n"/>
+      <c r="F15" s="3" t="n"/>
+      <c r="G15" s="3" t="n"/>
+      <c r="H15" s="3" t="n"/>
+      <c r="I15" s="3" t="n"/>
+      <c r="J15" s="3" t="n"/>
+      <c r="K15" s="18">
+        <f>SUM(K14:K14)</f>
+        <v/>
+      </c>
+      <c r="L15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>7.4</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Glycol circulation — pumps, tanks and controls</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7" t="n"/>
-      <c r="G11" s="7" t="n"/>
-      <c r="H11" s="7" t="n"/>
-      <c r="I11" s="7" t="n"/>
-      <c r="J11" s="7" t="n"/>
-      <c r="K11" s="7" t="n"/>
-      <c r="L11" s="7" t="n"/>
-    </row>
-    <row r="12">
-      <c r="B12" s="8" t="inlineStr">
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="7" t="n"/>
+      <c r="I16" s="7" t="n"/>
+      <c r="J16" s="7" t="n"/>
+      <c r="K16" s="7" t="n"/>
+      <c r="L16" s="7" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Glycol Pump</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>C-WP</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr"/>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr"/>
+      <c r="E17" s="10" t="inlineStr">
         <is>
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>RFQ</t>
         </is>
       </c>
-      <c r="G12" s="9" t="n">
+      <c r="G17" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="H12" s="9" t="inlineStr">
+      <c r="H17" s="9" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="I12" s="11" t="n"/>
-      <c r="J12" s="12" t="n">
+      <c r="I17" s="11" t="n"/>
+      <c r="J17" s="12" t="n">
         <v>0.15</v>
       </c>
-      <c r="K12" s="11">
-        <f>IFERROR($G12*$I12,"")</f>
-        <v/>
-      </c>
-      <c r="L12" s="13" t="inlineStr">
+      <c r="K17" s="11">
+        <f>IFERROR($G17*$I17,"")</f>
+        <v/>
+      </c>
+      <c r="L17" s="13" t="inlineStr">
         <is>
           <t>15 kW each · VSD</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="8" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Defrost Pump</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>C-WP</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr"/>
-      <c r="E13" s="10" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr"/>
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>RFQ</t>
         </is>
       </c>
-      <c r="G13" s="9" t="n">
+      <c r="G18" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H13" s="9" t="inlineStr">
+      <c r="H18" s="9" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="I13" s="11" t="n"/>
-      <c r="J13" s="12" t="n">
+      <c r="I18" s="11" t="n"/>
+      <c r="J18" s="12" t="n">
         <v>0.15</v>
       </c>
-      <c r="K13" s="11">
-        <f>IFERROR($G13*$I13,"")</f>
-        <v/>
-      </c>
-      <c r="L13" s="13" t="inlineStr">
+      <c r="K18" s="11">
+        <f>IFERROR($G18*$I18,"")</f>
+        <v/>
+      </c>
+      <c r="L18" s="13" t="inlineStr">
         <is>
           <t>4 kW each · VSD</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="n"/>
-      <c r="B14" s="3" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="3" t="n"/>
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Section 7.4 total</t>
         </is>
       </c>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
-      <c r="J14" s="3" t="n"/>
-      <c r="K14" s="14">
-        <f>SUM(K12:K13)</f>
-        <v/>
-      </c>
-      <c r="L14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="C19" s="3" t="n"/>
+      <c r="D19" s="3" t="n"/>
+      <c r="E19" s="3" t="n"/>
+      <c r="F19" s="3" t="n"/>
+      <c r="G19" s="3" t="n"/>
+      <c r="H19" s="3" t="n"/>
+      <c r="I19" s="3" t="n"/>
+      <c r="J19" s="3" t="n"/>
+      <c r="K19" s="18">
+        <f>SUM(K17:K18)</f>
+        <v/>
+      </c>
+      <c r="L19" s="3" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>7.5</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Unit coolers</t>
         </is>
       </c>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
-      <c r="F15" s="7" t="n"/>
-      <c r="G15" s="7" t="n"/>
-      <c r="H15" s="7" t="n"/>
-      <c r="I15" s="7" t="n"/>
-      <c r="J15" s="7" t="n"/>
-      <c r="K15" s="7" t="n"/>
-      <c r="L15" s="7" t="n"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="8" t="inlineStr">
+      <c r="C20" s="7" t="n"/>
+      <c r="D20" s="7" t="n"/>
+      <c r="E20" s="7" t="n"/>
+      <c r="F20" s="7" t="n"/>
+      <c r="G20" s="7" t="n"/>
+      <c r="H20" s="7" t="n"/>
+      <c r="I20" s="7" t="n"/>
+      <c r="J20" s="7" t="n"/>
+      <c r="K20" s="7" t="n"/>
+      <c r="L20" s="7" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>Unit Cooler</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>C-FCU</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr"/>
-      <c r="E16" s="10" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr"/>
+      <c r="E21" s="10" t="inlineStr">
         <is>
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>RFQ</t>
         </is>
       </c>
-      <c r="G16" s="9" t="n">
+      <c r="G21" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="H16" s="9" t="inlineStr">
+      <c r="H21" s="9" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="I16" s="11" t="n"/>
-      <c r="J16" s="12" t="n">
+      <c r="I21" s="11" t="n"/>
+      <c r="J21" s="12" t="n">
         <v>0.15</v>
       </c>
-      <c r="K16" s="11">
-        <f>IFERROR($G16*$I16,"")</f>
-        <v/>
-      </c>
-      <c r="L16" s="13" t="inlineStr">
+      <c r="K21" s="11">
+        <f>IFERROR($G21*$I21,"")</f>
+        <v/>
+      </c>
+      <c r="L21" s="13" t="inlineStr">
         <is>
           <t>55 kWR each · EC Fan Supply</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="n"/>
-      <c r="B17" s="3" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="3" t="n"/>
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Section 7.5 total</t>
         </is>
       </c>
-      <c r="C17" s="3" t="n"/>
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="n"/>
-      <c r="F17" s="3" t="n"/>
-      <c r="G17" s="3" t="n"/>
-      <c r="H17" s="3" t="n"/>
-      <c r="I17" s="3" t="n"/>
-      <c r="J17" s="3" t="n"/>
-      <c r="K17" s="14">
-        <f>SUM(K16:K16)</f>
-        <v/>
-      </c>
-      <c r="L17" s="3" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="C22" s="3" t="n"/>
+      <c r="D22" s="3" t="n"/>
+      <c r="E22" s="3" t="n"/>
+      <c r="F22" s="3" t="n"/>
+      <c r="G22" s="3" t="n"/>
+      <c r="H22" s="3" t="n"/>
+      <c r="I22" s="3" t="n"/>
+      <c r="J22" s="3" t="n"/>
+      <c r="K22" s="18">
+        <f>SUM(K21:K21)</f>
+        <v/>
+      </c>
+      <c r="L22" s="3" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>7.6</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Glycol pipework, valves and insulation</t>
         </is>
       </c>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
-      <c r="F18" s="7" t="n"/>
-      <c r="G18" s="7" t="n"/>
-      <c r="H18" s="7" t="n"/>
-      <c r="I18" s="7" t="n"/>
-      <c r="J18" s="7" t="n"/>
-      <c r="K18" s="7" t="n"/>
-      <c r="L18" s="7" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="15" t="inlineStr">
-        <is>
-          <t>50TE isolating valve</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>M-VG</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>BF-50TE</t>
-        </is>
-      </c>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="C23" s="7" t="n"/>
+      <c r="D23" s="7" t="n"/>
+      <c r="E23" s="7" t="n"/>
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="7" t="n"/>
+      <c r="H23" s="7" t="n"/>
+      <c r="I23" s="7" t="n"/>
+      <c r="J23" s="7" t="n"/>
+      <c r="K23" s="7" t="n"/>
+      <c r="L23" s="7" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>50TE tube flange</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>M-F</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr"/>
+      <c r="E24" s="10" t="inlineStr">
         <is>
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F19" s="16" t="inlineStr">
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>RULE</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="H24" s="10" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I24" s="20" t="n"/>
+      <c r="J24" s="21" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K24" s="20">
+        <f>IFERROR($G24*$I24,"")</f>
+        <v/>
+      </c>
+      <c r="L24" s="22" t="inlineStr">
+        <is>
+          <t>rule: 1 per 50TE connection</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>50TE gasket</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>M-F</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>GK-50</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>Bought in</t>
+        </is>
+      </c>
+      <c r="F25" s="15" t="inlineStr">
         <is>
           <t>PRICE LIST</t>
         </is>
       </c>
-      <c r="G19" t="n">
+      <c r="G25" t="n">
         <v>10</v>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="I19" s="17" t="n">
-        <v>84.5</v>
-      </c>
-      <c r="J19" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K19" s="4">
-        <f>IFERROR($G19*$I19,"")</f>
-        <v/>
-      </c>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
-          <t>10 × 50TE on the P&amp;ID</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="19" t="inlineStr">
-        <is>
-          <t>50TE tube flange</t>
-        </is>
-      </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>M-F</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr"/>
-      <c r="E20" s="10" t="inlineStr">
-        <is>
-          <t>Bought in</t>
-        </is>
-      </c>
-      <c r="F20" s="10" t="inlineStr">
-        <is>
-          <t>RULE</t>
-        </is>
-      </c>
-      <c r="G20" s="10" t="n">
-        <v>10</v>
-      </c>
-      <c r="H20" s="10" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I20" s="20" t="n"/>
-      <c r="J20" s="21" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K20" s="20">
-        <f>IFERROR($G20*$I20,"")</f>
-        <v/>
-      </c>
-      <c r="L20" s="22" t="inlineStr">
-        <is>
-          <t>rule: 1 per 50TE connection</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="15" t="inlineStr">
-        <is>
-          <t>50TE gasket</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>M-F</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>GK-50</t>
-        </is>
-      </c>
-      <c r="E21" s="10" t="inlineStr">
-        <is>
-          <t>Bought in</t>
-        </is>
-      </c>
-      <c r="F21" s="16" t="inlineStr">
-        <is>
-          <t>PRICE LIST</t>
-        </is>
-      </c>
-      <c r="G21" t="n">
-        <v>10</v>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I21" s="17" t="n">
+      <c r="I25" s="16" t="n">
         <v>4.8</v>
       </c>
-      <c r="J21" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K21" s="4">
-        <f>IFERROR($G21*$I21,"")</f>
-        <v/>
-      </c>
-      <c r="L21" s="2" t="inlineStr">
-        <is>
-          <t>rule: 1 per 50TE connection</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="15" t="inlineStr">
-        <is>
-          <t>80TE isolating valve</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>M-VG</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>BF-80TE</t>
-        </is>
-      </c>
-      <c r="E22" s="10" t="inlineStr">
-        <is>
-          <t>Bought in</t>
-        </is>
-      </c>
-      <c r="F22" s="16" t="inlineStr">
-        <is>
-          <t>PRICE LIST</t>
-        </is>
-      </c>
-      <c r="G22" t="n">
-        <v>6</v>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I22" s="17" t="n">
-        <v>112</v>
-      </c>
-      <c r="J22" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K22" s="4">
-        <f>IFERROR($G22*$I22,"")</f>
-        <v/>
-      </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>6 × 80TE on the P&amp;ID</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="19" t="inlineStr">
-        <is>
-          <t>80TE tube flange</t>
-        </is>
-      </c>
-      <c r="C23" s="10" t="inlineStr">
-        <is>
-          <t>M-F</t>
-        </is>
-      </c>
-      <c r="D23" s="10" t="inlineStr"/>
-      <c r="E23" s="10" t="inlineStr">
-        <is>
-          <t>Bought in</t>
-        </is>
-      </c>
-      <c r="F23" s="10" t="inlineStr">
-        <is>
-          <t>RULE</t>
-        </is>
-      </c>
-      <c r="G23" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="H23" s="10" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I23" s="20" t="n"/>
-      <c r="J23" s="21" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K23" s="20">
-        <f>IFERROR($G23*$I23,"")</f>
-        <v/>
-      </c>
-      <c r="L23" s="22" t="inlineStr">
-        <is>
-          <t>rule: 1 per 80TE connection</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="15" t="inlineStr">
-        <is>
-          <t>80TE gasket</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>M-F</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>GK-80</t>
-        </is>
-      </c>
-      <c r="E24" s="10" t="inlineStr">
-        <is>
-          <t>Bought in</t>
-        </is>
-      </c>
-      <c r="F24" s="16" t="inlineStr">
-        <is>
-          <t>PRICE LIST</t>
-        </is>
-      </c>
-      <c r="G24" t="n">
-        <v>6</v>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I24" s="17" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="J24" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K24" s="4">
-        <f>IFERROR($G24*$I24,"")</f>
-        <v/>
-      </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>rule: 1 per 80TE connection</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="15" t="inlineStr">
-        <is>
-          <t>40PN isolating valve</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>M-VG</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>BF-40PN</t>
-        </is>
-      </c>
-      <c r="E25" s="10" t="inlineStr">
-        <is>
-          <t>Bought in</t>
-        </is>
-      </c>
-      <c r="F25" s="16" t="inlineStr">
-        <is>
-          <t>PRICE LIST</t>
-        </is>
-      </c>
-      <c r="G25" t="n">
-        <v>2</v>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I25" s="17" t="n">
-        <v>121</v>
-      </c>
-      <c r="J25" s="18" t="n">
+      <c r="J25" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K25" s="4">
@@ -1581,142 +1587,142 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>2 × 40PN on the P&amp;ID</t>
+          <t>rule: 1 per 50TE connection</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="15" t="inlineStr">
+      <c r="B26" s="19" t="inlineStr">
+        <is>
+          <t>80TE tube flange</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>M-F</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="inlineStr"/>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>Bought in</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>RULE</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="H26" s="10" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I26" s="20" t="n"/>
+      <c r="J26" s="21" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K26" s="20">
+        <f>IFERROR($G26*$I26,"")</f>
+        <v/>
+      </c>
+      <c r="L26" s="22" t="inlineStr">
+        <is>
+          <t>rule: 1 per 80TE connection</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>80TE gasket</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>M-F</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>GK-80</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>Bought in</t>
+        </is>
+      </c>
+      <c r="F27" s="15" t="inlineStr">
+        <is>
+          <t>PRICE LIST</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>6</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I27" s="16" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="J27" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K27" s="4">
+        <f>IFERROR($G27*$I27,"")</f>
+        <v/>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>rule: 1 per 80TE connection</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="14" t="inlineStr">
         <is>
           <t>40PN gasket</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>M-F</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>GK-40</t>
         </is>
       </c>
-      <c r="E26" s="10" t="inlineStr">
+      <c r="E28" s="10" t="inlineStr">
         <is>
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F26" s="16" t="inlineStr">
+      <c r="F28" s="15" t="inlineStr">
         <is>
           <t>PRICE LIST</t>
         </is>
       </c>
-      <c r="G26" t="n">
+      <c r="G28" t="n">
         <v>2</v>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="I26" s="17" t="n">
+      <c r="I28" s="16" t="n">
         <v>3.9</v>
       </c>
-      <c r="J26" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K26" s="4">
-        <f>IFERROR($G26*$I26,"")</f>
-        <v/>
-      </c>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>rule: 1 per 40PN connection</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="19" t="inlineStr">
-        <is>
-          <t>40PN bolt set</t>
-        </is>
-      </c>
-      <c r="C27" s="10" t="inlineStr">
-        <is>
-          <t>M-F</t>
-        </is>
-      </c>
-      <c r="D27" s="10" t="inlineStr"/>
-      <c r="E27" s="10" t="inlineStr">
-        <is>
-          <t>Bought in</t>
-        </is>
-      </c>
-      <c r="F27" s="10" t="inlineStr">
-        <is>
-          <t>RULE</t>
-        </is>
-      </c>
-      <c r="G27" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="H27" s="10" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I27" s="20" t="n"/>
-      <c r="J27" s="21" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K27" s="20">
-        <f>IFERROR($G27*$I27,"")</f>
-        <v/>
-      </c>
-      <c r="L27" s="22" t="inlineStr">
-        <is>
-          <t>rule: 1 per 40PN connection</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="15" t="inlineStr">
-        <is>
-          <t>65PN isolating valve</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>M-VG</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>BF-65PN</t>
-        </is>
-      </c>
-      <c r="E28" s="10" t="inlineStr">
-        <is>
-          <t>Bought in</t>
-        </is>
-      </c>
-      <c r="F28" s="16" t="inlineStr">
-        <is>
-          <t>PRICE LIST</t>
-        </is>
-      </c>
-      <c r="G28" t="n">
-        <v>1</v>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I28" s="17" t="n">
-        <v>168</v>
-      </c>
-      <c r="J28" s="18" t="n">
+      <c r="J28" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K28" s="4">
@@ -1725,151 +1731,145 @@
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>1 × 65PN on the P&amp;ID</t>
+          <t>rule: 1 per 40PN connection</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="15" t="inlineStr">
+      <c r="B29" s="19" t="inlineStr">
+        <is>
+          <t>40PN bolt set</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>M-F</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr"/>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>Bought in</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>RULE</t>
+        </is>
+      </c>
+      <c r="G29" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" s="10" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I29" s="20" t="n"/>
+      <c r="J29" s="21" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K29" s="20">
+        <f>IFERROR($G29*$I29,"")</f>
+        <v/>
+      </c>
+      <c r="L29" s="22" t="inlineStr">
+        <is>
+          <t>rule: 1 per 40PN connection</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="14" t="inlineStr">
         <is>
           <t>65PN gasket</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>M-F</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>GK-65</t>
         </is>
       </c>
-      <c r="E29" s="10" t="inlineStr">
+      <c r="E30" s="10" t="inlineStr">
         <is>
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F29" s="16" t="inlineStr">
+      <c r="F30" s="15" t="inlineStr">
         <is>
           <t>PRICE LIST</t>
         </is>
       </c>
-      <c r="G29" t="n">
+      <c r="G30" t="n">
         <v>1</v>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="I29" s="17" t="n">
+      <c r="I30" s="16" t="n">
         <v>5.4</v>
       </c>
-      <c r="J29" s="18" t="n">
+      <c r="J30" s="17" t="n">
         <v>0.15</v>
       </c>
-      <c r="K29" s="4">
-        <f>IFERROR($G29*$I29,"")</f>
-        <v/>
-      </c>
-      <c r="L29" s="2" t="inlineStr">
+      <c r="K30" s="4">
+        <f>IFERROR($G30*$I30,"")</f>
+        <v/>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
         <is>
           <t>rule: 1 per 65PN connection</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="B30" s="19" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="19" t="inlineStr">
         <is>
           <t>65PN bolt set</t>
         </is>
       </c>
-      <c r="C30" s="10" t="inlineStr">
+      <c r="C31" s="10" t="inlineStr">
         <is>
           <t>M-F</t>
         </is>
       </c>
-      <c r="D30" s="10" t="inlineStr"/>
-      <c r="E30" s="10" t="inlineStr">
+      <c r="D31" s="10" t="inlineStr"/>
+      <c r="E31" s="10" t="inlineStr">
         <is>
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F30" s="10" t="inlineStr">
+      <c r="F31" s="10" t="inlineStr">
         <is>
           <t>RULE</t>
         </is>
       </c>
-      <c r="G30" s="10" t="n">
+      <c r="G31" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H30" s="10" t="inlineStr">
+      <c r="H31" s="10" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="I30" s="20" t="n"/>
-      <c r="J30" s="21" t="n">
+      <c r="I31" s="20" t="n"/>
+      <c r="J31" s="21" t="n">
         <v>0.15</v>
       </c>
-      <c r="K30" s="20">
-        <f>IFERROR($G30*$I30,"")</f>
-        <v/>
-      </c>
-      <c r="L30" s="22" t="inlineStr">
+      <c r="K31" s="20">
+        <f>IFERROR($G31*$I31,"")</f>
+        <v/>
+      </c>
+      <c r="L31" s="22" t="inlineStr">
         <is>
           <t>rule: 1 per 65PN connection</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="15" t="inlineStr">
-        <is>
-          <t>65TE isolating valve</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>M-VG</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>BF-65TE</t>
-        </is>
-      </c>
-      <c r="E31" s="10" t="inlineStr">
-        <is>
-          <t>Bought in</t>
-        </is>
-      </c>
-      <c r="F31" s="16" t="inlineStr">
-        <is>
-          <t>PRICE LIST</t>
-        </is>
-      </c>
-      <c r="G31" t="n">
-        <v>1</v>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I31" s="17" t="n">
-        <v>138</v>
-      </c>
-      <c r="J31" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K31" s="4">
-        <f>IFERROR($G31*$I31,"")</f>
-        <v/>
-      </c>
-      <c r="L31" s="2" t="inlineStr">
-        <is>
-          <t>1 × 65TE on the P&amp;ID</t>
         </is>
       </c>
     </row>
@@ -1918,7 +1918,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="15" t="inlineStr">
+      <c r="B33" s="14" t="inlineStr">
         <is>
           <t>65TE gasket</t>
         </is>
@@ -1938,7 +1938,7 @@
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F33" s="16" t="inlineStr">
+      <c r="F33" s="15" t="inlineStr">
         <is>
           <t>PRICE LIST</t>
         </is>
@@ -1951,10 +1951,10 @@
           <t>ea</t>
         </is>
       </c>
-      <c r="I33" s="17" t="n">
+      <c r="I33" s="16" t="n">
         <v>5.4</v>
       </c>
-      <c r="J33" s="18" t="n">
+      <c r="J33" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K33" s="4">
@@ -1968,7 +1968,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="15" t="inlineStr">
+      <c r="B34" s="14" t="inlineStr">
         <is>
           <t>42mm 304 press pipe</t>
         </is>
@@ -1988,7 +1988,7 @@
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F34" s="16" t="inlineStr">
+      <c r="F34" s="15" t="inlineStr">
         <is>
           <t>PRICE LIST</t>
         </is>
@@ -1998,10 +1998,10 @@
           <t>m</t>
         </is>
       </c>
-      <c r="I34" s="17" t="n">
+      <c r="I34" s="16" t="n">
         <v>11.9</v>
       </c>
-      <c r="J34" s="18" t="n">
+      <c r="J34" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K34" s="4">
@@ -2015,7 +2015,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="15" t="inlineStr">
+      <c r="B35" s="14" t="inlineStr">
         <is>
           <t>100NB pipe</t>
         </is>
@@ -2042,7 +2042,7 @@
         </is>
       </c>
       <c r="I35" s="4" t="n"/>
-      <c r="J35" s="18" t="n">
+      <c r="J35" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K35" s="4">
@@ -2056,7 +2056,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="15" t="inlineStr">
+      <c r="B36" s="14" t="inlineStr">
         <is>
           <t>80NB pipe</t>
         </is>
@@ -2083,7 +2083,7 @@
         </is>
       </c>
       <c r="I36" s="4" t="n"/>
-      <c r="J36" s="18" t="n">
+      <c r="J36" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K36" s="4">
@@ -2097,7 +2097,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="15" t="inlineStr">
+      <c r="B37" s="14" t="inlineStr">
         <is>
           <t>101mm tube pipe</t>
         </is>
@@ -2124,7 +2124,7 @@
         </is>
       </c>
       <c r="I37" s="4" t="n"/>
-      <c r="J37" s="18" t="n">
+      <c r="J37" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K37" s="4">
@@ -2138,7 +2138,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="15" t="inlineStr">
+      <c r="B38" s="14" t="inlineStr">
         <is>
           <t>63mm tube pipe</t>
         </is>
@@ -2165,7 +2165,7 @@
         </is>
       </c>
       <c r="I38" s="4" t="n"/>
-      <c r="J38" s="18" t="n">
+      <c r="J38" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K38" s="4">
@@ -2179,7 +2179,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="15" t="inlineStr">
+      <c r="B39" s="14" t="inlineStr">
         <is>
           <t>76mm 304 press pipe</t>
         </is>
@@ -2199,7 +2199,7 @@
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F39" s="16" t="inlineStr">
+      <c r="F39" s="15" t="inlineStr">
         <is>
           <t>PRICE LIST</t>
         </is>
@@ -2209,10 +2209,10 @@
           <t>m</t>
         </is>
       </c>
-      <c r="I39" s="17" t="n">
+      <c r="I39" s="16" t="n">
         <v>53.1</v>
       </c>
-      <c r="J39" s="18" t="n">
+      <c r="J39" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K39" s="4">
@@ -2226,7 +2226,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="15" t="inlineStr">
+      <c r="B40" s="14" t="inlineStr">
         <is>
           <t>54mm 304 press pipe</t>
         </is>
@@ -2246,7 +2246,7 @@
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F40" s="16" t="inlineStr">
+      <c r="F40" s="15" t="inlineStr">
         <is>
           <t>PRICE LIST</t>
         </is>
@@ -2256,10 +2256,10 @@
           <t>m</t>
         </is>
       </c>
-      <c r="I40" s="17" t="n">
+      <c r="I40" s="16" t="n">
         <v>17.4</v>
       </c>
-      <c r="J40" s="18" t="n">
+      <c r="J40" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K40" s="4">
@@ -2315,7 +2315,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="15" t="inlineStr">
+      <c r="B42" s="14" t="inlineStr">
         <is>
           <t>Freight and cartage</t>
         </is>
@@ -2342,7 +2342,7 @@
         </is>
       </c>
       <c r="I42" s="4" t="n"/>
-      <c r="J42" s="18" t="n">
+      <c r="J42" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K42" s="4">
@@ -2370,8 +2370,8 @@
       <c r="H43" s="3" t="n"/>
       <c r="I43" s="3" t="n"/>
       <c r="J43" s="3" t="n"/>
-      <c r="K43" s="14">
-        <f>SUM(K19:K42)</f>
+      <c r="K43" s="18">
+        <f>SUM(K24:K42)</f>
         <v/>
       </c>
       <c r="L43" s="3" t="n"/>
@@ -2399,7 +2399,7 @@
       <c r="L44" s="7" t="n"/>
     </row>
     <row r="45">
-      <c r="B45" s="15" t="inlineStr">
+      <c r="B45" s="14" t="inlineStr">
         <is>
           <t>Set out and rig plant</t>
         </is>
@@ -2410,7 +2410,7 @@
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
-      <c r="E45" s="16" t="inlineStr">
+      <c r="E45" s="15" t="inlineStr">
         <is>
           <t>In-house</t>
         </is>
@@ -2428,7 +2428,7 @@
       <c r="I45" s="4" t="n">
         <v>105</v>
       </c>
-      <c r="J45" s="18" t="n">
+      <c r="J45" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K45" s="4">
@@ -2442,7 +2442,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="B46" s="15" t="inlineStr">
+      <c r="B46" s="14" t="inlineStr">
         <is>
           <t>Pipe compressor pack</t>
         </is>
@@ -2453,7 +2453,7 @@
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
-      <c r="E46" s="16" t="inlineStr">
+      <c r="E46" s="15" t="inlineStr">
         <is>
           <t>In-house</t>
         </is>
@@ -2471,7 +2471,7 @@
       <c r="I46" s="4" t="n">
         <v>105</v>
       </c>
-      <c r="J46" s="18" t="n">
+      <c r="J46" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K46" s="4">
@@ -2485,7 +2485,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="B47" s="15" t="inlineStr">
+      <c r="B47" s="14" t="inlineStr">
         <is>
           <t>Pipe chiller and glycol circuit</t>
         </is>
@@ -2496,7 +2496,7 @@
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
-      <c r="E47" s="16" t="inlineStr">
+      <c r="E47" s="15" t="inlineStr">
         <is>
           <t>In-house</t>
         </is>
@@ -2514,7 +2514,7 @@
       <c r="I47" s="4" t="n">
         <v>105</v>
       </c>
-      <c r="J47" s="18" t="n">
+      <c r="J47" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K47" s="4">
@@ -2528,7 +2528,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="B48" s="15" t="inlineStr">
+      <c r="B48" s="14" t="inlineStr">
         <is>
           <t>Hang and pipe unit coolers</t>
         </is>
@@ -2539,7 +2539,7 @@
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
-      <c r="E48" s="16" t="inlineStr">
+      <c r="E48" s="15" t="inlineStr">
         <is>
           <t>In-house</t>
         </is>
@@ -2557,7 +2557,7 @@
       <c r="I48" s="4" t="n">
         <v>105</v>
       </c>
-      <c r="J48" s="18" t="n">
+      <c r="J48" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K48" s="4">
@@ -2571,7 +2571,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="B49" s="15" t="inlineStr">
+      <c r="B49" s="14" t="inlineStr">
         <is>
           <t>Pressure test</t>
         </is>
@@ -2582,7 +2582,7 @@
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
-      <c r="E49" s="16" t="inlineStr">
+      <c r="E49" s="15" t="inlineStr">
         <is>
           <t>In-house</t>
         </is>
@@ -2600,7 +2600,7 @@
       <c r="I49" s="4" t="n">
         <v>105</v>
       </c>
-      <c r="J49" s="18" t="n">
+      <c r="J49" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K49" s="4">
@@ -2614,7 +2614,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="B50" s="15" t="inlineStr">
+      <c r="B50" s="14" t="inlineStr">
         <is>
           <t>Insulate</t>
         </is>
@@ -2625,7 +2625,7 @@
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
-      <c r="E50" s="16" t="inlineStr">
+      <c r="E50" s="15" t="inlineStr">
         <is>
           <t>In-house</t>
         </is>
@@ -2643,7 +2643,7 @@
       <c r="I50" s="4" t="n">
         <v>105</v>
       </c>
-      <c r="J50" s="18" t="n">
+      <c r="J50" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K50" s="4">
@@ -2657,7 +2657,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="B51" s="15" t="inlineStr">
+      <c r="B51" s="14" t="inlineStr">
         <is>
           <t>Glycol fill and flush</t>
         </is>
@@ -2668,7 +2668,7 @@
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
-      <c r="E51" s="16" t="inlineStr">
+      <c r="E51" s="15" t="inlineStr">
         <is>
           <t>In-house</t>
         </is>
@@ -2686,7 +2686,7 @@
       <c r="I51" s="4" t="n">
         <v>105</v>
       </c>
-      <c r="J51" s="18" t="n">
+      <c r="J51" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K51" s="4">
@@ -2700,7 +2700,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="B52" s="15" t="inlineStr">
+      <c r="B52" s="14" t="inlineStr">
         <is>
           <t>Changeover weekend</t>
         </is>
@@ -2711,7 +2711,7 @@
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
-      <c r="E52" s="16" t="inlineStr">
+      <c r="E52" s="15" t="inlineStr">
         <is>
           <t>In-house</t>
         </is>
@@ -2729,7 +2729,7 @@
       <c r="I52" s="4" t="n">
         <v>105</v>
       </c>
-      <c r="J52" s="18" t="n">
+      <c r="J52" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K52" s="4">
@@ -2743,7 +2743,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="B53" s="15" t="inlineStr">
+      <c r="B53" s="14" t="inlineStr">
         <is>
           <t>Supervision</t>
         </is>
@@ -2754,7 +2754,7 @@
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
-      <c r="E53" s="16" t="inlineStr">
+      <c r="E53" s="15" t="inlineStr">
         <is>
           <t>In-house</t>
         </is>
@@ -2772,7 +2772,7 @@
       <c r="I53" s="4" t="n">
         <v>105</v>
       </c>
-      <c r="J53" s="18" t="n">
+      <c r="J53" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K53" s="4">
@@ -2786,7 +2786,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="B54" s="15" t="inlineStr">
+      <c r="B54" s="14" t="inlineStr">
         <is>
           <t>Crane and access hire</t>
         </is>
@@ -2813,7 +2813,7 @@
         </is>
       </c>
       <c r="I54" s="4" t="n"/>
-      <c r="J54" s="18" t="n">
+      <c r="J54" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K54" s="4">
@@ -2827,7 +2827,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="B55" s="15" t="inlineStr">
+      <c r="B55" s="14" t="inlineStr">
         <is>
           <t>Travel and accommodation</t>
         </is>
@@ -2854,7 +2854,7 @@
         </is>
       </c>
       <c r="I55" s="4" t="n"/>
-      <c r="J55" s="18" t="n">
+      <c r="J55" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K55" s="4">
@@ -2868,7 +2868,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="B56" s="15" t="inlineStr">
+      <c r="B56" s="14" t="inlineStr">
         <is>
           <t>Site setup and safety</t>
         </is>
@@ -2895,7 +2895,7 @@
         </is>
       </c>
       <c r="I56" s="4" t="n"/>
-      <c r="J56" s="18" t="n">
+      <c r="J56" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K56" s="4">
@@ -2909,23 +2909,23 @@
       </c>
     </row>
     <row r="57">
-      <c r="B57" s="16" t="inlineStr">
+      <c r="B57" s="15" t="inlineStr">
         <is>
           <t>Site welding and fit-up</t>
         </is>
       </c>
-      <c r="C57" s="16" t="inlineStr">
+      <c r="C57" s="15" t="inlineStr">
         <is>
           <t>L-SERVIN</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
-      <c r="E57" s="16" t="inlineStr">
+      <c r="E57" s="15" t="inlineStr">
         <is>
           <t>In-house</t>
         </is>
       </c>
-      <c r="F57" s="16" t="inlineStr">
+      <c r="F57" s="15" t="inlineStr">
         <is>
           <t>TAKE-OFF</t>
         </is>
@@ -2934,18 +2934,18 @@
         <f>'Take-off'!F20</f>
         <v/>
       </c>
-      <c r="H57" s="16" t="inlineStr">
+      <c r="H57" s="15" t="inlineStr">
         <is>
           <t>hr</t>
         </is>
       </c>
-      <c r="I57" s="17" t="n">
+      <c r="I57" s="16" t="n">
         <v>110</v>
       </c>
       <c r="J57" s="24" t="n">
         <v>0.15</v>
       </c>
-      <c r="K57" s="17">
+      <c r="K57" s="16">
         <f>IFERROR($G57*$I57,"")</f>
         <v/>
       </c>
@@ -2970,7 +2970,7 @@
       <c r="H58" s="3" t="n"/>
       <c r="I58" s="3" t="n"/>
       <c r="J58" s="3" t="n"/>
-      <c r="K58" s="14">
+      <c r="K58" s="18">
         <f>SUM(K45:K57)</f>
         <v/>
       </c>
@@ -3101,7 +3101,7 @@
       <c r="H62" s="3" t="n"/>
       <c r="I62" s="3" t="n"/>
       <c r="J62" s="3" t="n"/>
-      <c r="K62" s="14">
+      <c r="K62" s="18">
         <f>SUM(K60:K61)</f>
         <v/>
       </c>
@@ -3130,7 +3130,7 @@
       <c r="L63" s="7" t="n"/>
     </row>
     <row r="64">
-      <c r="B64" s="15" t="inlineStr">
+      <c r="B64" s="14" t="inlineStr">
         <is>
           <t>As-built drawings</t>
         </is>
@@ -3141,7 +3141,7 @@
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
-      <c r="E64" s="16" t="inlineStr">
+      <c r="E64" s="15" t="inlineStr">
         <is>
           <t>In-house</t>
         </is>
@@ -3159,7 +3159,7 @@
       <c r="I64" s="4" t="n">
         <v>140</v>
       </c>
-      <c r="J64" s="18" t="n">
+      <c r="J64" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K64" s="4">
@@ -3173,7 +3173,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="B65" s="15" t="inlineStr">
+      <c r="B65" s="14" t="inlineStr">
         <is>
           <t>Training</t>
         </is>
@@ -3184,7 +3184,7 @@
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
-      <c r="E65" s="16" t="inlineStr">
+      <c r="E65" s="15" t="inlineStr">
         <is>
           <t>In-house</t>
         </is>
@@ -3202,7 +3202,7 @@
       <c r="I65" s="4" t="n">
         <v>140</v>
       </c>
-      <c r="J65" s="18" t="n">
+      <c r="J65" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K65" s="4">
@@ -3216,7 +3216,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="B66" s="15" t="inlineStr">
+      <c r="B66" s="14" t="inlineStr">
         <is>
           <t>O&amp;M manuals</t>
         </is>
@@ -3227,7 +3227,7 @@
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
-      <c r="E66" s="16" t="inlineStr">
+      <c r="E66" s="15" t="inlineStr">
         <is>
           <t>In-house</t>
         </is>
@@ -3245,7 +3245,7 @@
       <c r="I66" s="4" t="n">
         <v>140</v>
       </c>
-      <c r="J66" s="18" t="n">
+      <c r="J66" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K66" s="4">
@@ -3259,7 +3259,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="B67" s="15" t="inlineStr">
+      <c r="B67" s="14" t="inlineStr">
         <is>
           <t>Producer statements</t>
         </is>
@@ -3270,7 +3270,7 @@
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
-      <c r="E67" s="16" t="inlineStr">
+      <c r="E67" s="15" t="inlineStr">
         <is>
           <t>In-house</t>
         </is>
@@ -3288,7 +3288,7 @@
       <c r="I67" s="4" t="n">
         <v>140</v>
       </c>
-      <c r="J67" s="18" t="n">
+      <c r="J67" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K67" s="4">
@@ -3302,7 +3302,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="B68" s="15" t="inlineStr">
+      <c r="B68" s="14" t="inlineStr">
         <is>
           <t>Compliance and inspection</t>
         </is>
@@ -3329,7 +3329,7 @@
         </is>
       </c>
       <c r="I68" s="4" t="n"/>
-      <c r="J68" s="18" t="n">
+      <c r="J68" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K68" s="4">
@@ -3357,7 +3357,7 @@
       <c r="H69" s="3" t="n"/>
       <c r="I69" s="3" t="n"/>
       <c r="J69" s="3" t="n"/>
-      <c r="K69" s="14">
+      <c r="K69" s="18">
         <f>SUM(K64:K68)</f>
         <v/>
       </c>
@@ -3386,7 +3386,7 @@
       <c r="L70" s="7" t="n"/>
     </row>
     <row r="71">
-      <c r="B71" s="15" t="inlineStr">
+      <c r="B71" s="14" t="inlineStr">
         <is>
           <t>Commissioning and pulldown demonstration</t>
         </is>
@@ -3397,7 +3397,7 @@
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
-      <c r="E71" s="16" t="inlineStr">
+      <c r="E71" s="15" t="inlineStr">
         <is>
           <t>In-house</t>
         </is>
@@ -3415,7 +3415,7 @@
       <c r="I71" s="4" t="n">
         <v>105</v>
       </c>
-      <c r="J71" s="18" t="n">
+      <c r="J71" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K71" s="4">
@@ -3429,7 +3429,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="B72" s="15" t="inlineStr">
+      <c r="B72" s="14" t="inlineStr">
         <is>
           <t>Glycol charge — MPG 35%</t>
         </is>
@@ -3456,7 +3456,7 @@
         </is>
       </c>
       <c r="I72" s="4" t="n"/>
-      <c r="J72" s="18" t="n">
+      <c r="J72" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K72" s="4">
@@ -3470,7 +3470,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="B73" s="15" t="inlineStr">
+      <c r="B73" s="14" t="inlineStr">
         <is>
           <t>Spare parts</t>
         </is>
@@ -3497,7 +3497,7 @@
         </is>
       </c>
       <c r="I73" s="4" t="n"/>
-      <c r="J73" s="18" t="n">
+      <c r="J73" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K73" s="4">
@@ -3525,7 +3525,7 @@
       <c r="H74" s="3" t="n"/>
       <c r="I74" s="3" t="n"/>
       <c r="J74" s="3" t="n"/>
-      <c r="K74" s="14">
+      <c r="K74" s="18">
         <f>SUM(K71:K73)</f>
         <v/>
       </c>
@@ -3554,7 +3554,7 @@
       <c r="L75" s="7" t="n"/>
     </row>
     <row r="76">
-      <c r="B76" s="15" t="inlineStr">
+      <c r="B76" s="14" t="inlineStr">
         <is>
           <t>Routine maintenance, 12 months</t>
         </is>
@@ -3584,7 +3584,7 @@
         </is>
       </c>
       <c r="I76" s="4" t="n"/>
-      <c r="J76" s="18" t="n">
+      <c r="J76" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K76" s="4">
@@ -3598,7 +3598,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="B77" s="15" t="inlineStr">
+      <c r="B77" s="14" t="inlineStr">
         <is>
           <t>Contingency</t>
         </is>
@@ -3625,7 +3625,7 @@
         </is>
       </c>
       <c r="I77" s="4" t="n"/>
-      <c r="J77" s="18" t="n">
+      <c r="J77" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="K77" s="4">
@@ -3653,7 +3653,7 @@
       <c r="H78" s="3" t="n"/>
       <c r="I78" s="3" t="n"/>
       <c r="J78" s="3" t="n"/>
-      <c r="K78" s="14">
+      <c r="K78" s="18">
         <f>SUM(K76:K77)</f>
         <v/>
       </c>
@@ -3674,8 +3674,8 @@
       <c r="H80" s="3" t="n"/>
       <c r="I80" s="3" t="n"/>
       <c r="J80" s="3" t="n"/>
-      <c r="K80" s="14">
-        <f>K4+K7+K10+K14+K17+K43+K58+K62+K69+K74+K78</f>
+      <c r="K80" s="18">
+        <f>K9+K12+K15+K19+K22+K43+K58+K62+K69+K74+K78</f>
         <v/>
       </c>
       <c r="L80" s="3" t="n"/>
@@ -3745,10 +3745,10 @@
         </is>
       </c>
       <c r="C2" s="4">
-        <f>Costing!K4</f>
-        <v/>
-      </c>
-      <c r="D2" s="18" t="n">
+        <f>Costing!K9</f>
+        <v/>
+      </c>
+      <c r="D2" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="E2" s="4">
@@ -3768,10 +3768,10 @@
         </is>
       </c>
       <c r="C3" s="4">
-        <f>Costing!K7</f>
-        <v/>
-      </c>
-      <c r="D3" s="18" t="n">
+        <f>Costing!K12</f>
+        <v/>
+      </c>
+      <c r="D3" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="E3" s="4">
@@ -3791,10 +3791,10 @@
         </is>
       </c>
       <c r="C4" s="4">
-        <f>Costing!K10</f>
-        <v/>
-      </c>
-      <c r="D4" s="18" t="n">
+        <f>Costing!K15</f>
+        <v/>
+      </c>
+      <c r="D4" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="E4" s="4">
@@ -3814,10 +3814,10 @@
         </is>
       </c>
       <c r="C5" s="4">
-        <f>Costing!K14</f>
-        <v/>
-      </c>
-      <c r="D5" s="18" t="n">
+        <f>Costing!K19</f>
+        <v/>
+      </c>
+      <c r="D5" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="E5" s="4">
@@ -3837,10 +3837,10 @@
         </is>
       </c>
       <c r="C6" s="4">
-        <f>Costing!K17</f>
-        <v/>
-      </c>
-      <c r="D6" s="18" t="n">
+        <f>Costing!K22</f>
+        <v/>
+      </c>
+      <c r="D6" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="E6" s="4">
@@ -3863,7 +3863,7 @@
         <f>Costing!K43</f>
         <v/>
       </c>
-      <c r="D7" s="18" t="n">
+      <c r="D7" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="E7" s="4">
@@ -3886,7 +3886,7 @@
         <f>Costing!K58</f>
         <v/>
       </c>
-      <c r="D8" s="18" t="n">
+      <c r="D8" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="E8" s="4">
@@ -3909,7 +3909,7 @@
         <f>Costing!K62</f>
         <v/>
       </c>
-      <c r="D9" s="18" t="n">
+      <c r="D9" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="E9" s="4">
@@ -3932,7 +3932,7 @@
         <f>Costing!K69</f>
         <v/>
       </c>
-      <c r="D10" s="18" t="n">
+      <c r="D10" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="E10" s="4">
@@ -3955,7 +3955,7 @@
         <f>Costing!K74</f>
         <v/>
       </c>
-      <c r="D11" s="18" t="n">
+      <c r="D11" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="E11" s="4">
@@ -3978,7 +3978,7 @@
         <f>Costing!K78</f>
         <v/>
       </c>
-      <c r="D12" s="18" t="n">
+      <c r="D12" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="E12" s="4">
@@ -3993,12 +3993,12 @@
           <t>Total (excl GST)</t>
         </is>
       </c>
-      <c r="C14" s="14">
+      <c r="C14" s="18">
         <f>SUM(C2:C12)</f>
         <v/>
       </c>
       <c r="D14" s="3" t="n"/>
-      <c r="E14" s="14">
+      <c r="E14" s="18">
         <f>SUM(E2:E12)</f>
         <v/>
       </c>
@@ -4023,7 +4023,7 @@
       </c>
       <c r="C16" s="3" t="n"/>
       <c r="D16" s="3" t="n"/>
-      <c r="E16" s="14">
+      <c r="E16" s="18">
         <f>E14+E15</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
quote-builder: run lengths read off the P&ID -> pipe, insulation, welding (Riverbend-Q900142-Costing.xlsx)
</commit_message>
<xml_diff>
--- a/quote-builder/Riverbend-Q900142-Costing.xlsx
+++ b/quote-builder/Riverbend-Q900142-Costing.xlsx
@@ -70,12 +70,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF4E0"/>
+        <fgColor rgb="00DCE6F1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCE6F1"/>
+        <fgColor rgb="00FFF4E0"/>
       </patternFill>
     </fill>
     <fill>
@@ -101,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -111,12 +111,12 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -127,17 +127,16 @@
     <xf numFmtId="4" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -567,7 +566,7 @@
         </is>
       </c>
       <c r="B8" s="4">
-        <f>Costing!K80</f>
+        <f>Costing!K81</f>
         <v/>
       </c>
     </row>
@@ -623,7 +622,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15">
@@ -667,7 +666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L80"/>
+  <dimension ref="A1:L81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -839,7 +838,7 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -858,7 +857,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>10 × 50TE on the P&amp;ID</t>
+          <t>9 × 50TE on the P&amp;ID</t>
         </is>
       </c>
     </row>
@@ -889,7 +888,7 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -908,7 +907,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>6 × 80TE on the P&amp;ID</t>
+          <t>4 × 80TE on the P&amp;ID</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1519,7 @@
         </is>
       </c>
       <c r="G24" s="10" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H24" s="10" t="inlineStr">
         <is>
@@ -1568,7 +1567,7 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -1614,7 +1613,7 @@
         </is>
       </c>
       <c r="G26" s="10" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H26" s="10" t="inlineStr">
         <is>
@@ -1662,7 +1661,7 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -1993,6 +1992,9 @@
           <t>PRICE LIST</t>
         </is>
       </c>
+      <c r="G34" t="n">
+        <v>48</v>
+      </c>
       <c r="H34" t="inlineStr">
         <is>
           <t>m</t>
@@ -2010,14 +2012,14 @@
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>8 runs on the P&amp;ID — metres not on the drawing</t>
+          <t>8 runs on the P&amp;ID · 6 m ×8 off the drawing = 48 m</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="14" t="inlineStr">
         <is>
-          <t>100NB pipe</t>
+          <t>80NB pipe</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2036,6 +2038,9 @@
           <t>ENGINEER</t>
         </is>
       </c>
+      <c r="G35" t="n">
+        <v>98</v>
+      </c>
       <c r="H35" t="inlineStr">
         <is>
           <t>m</t>
@@ -2051,14 +2056,14 @@
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>1 runs on the P&amp;ID — metres not on the drawing</t>
+          <t>3 runs on the P&amp;ID · 8 + 45 + 45 m off the drawing = 98 m</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="14" t="inlineStr">
         <is>
-          <t>80NB pipe</t>
+          <t>100NB pipe</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2077,6 +2082,9 @@
           <t>ENGINEER</t>
         </is>
       </c>
+      <c r="G36" t="n">
+        <v>8</v>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
           <t>m</t>
@@ -2092,14 +2100,14 @@
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>1 runs on the P&amp;ID — metres not on the drawing</t>
+          <t>1 run on the P&amp;ID · 8 m off the drawing = 8 m</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="14" t="inlineStr">
         <is>
-          <t>101mm tube pipe</t>
+          <t>50NB pipe</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2118,6 +2126,9 @@
           <t>ENGINEER</t>
         </is>
       </c>
+      <c r="G37" t="n">
+        <v>45</v>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
           <t>m</t>
@@ -2133,14 +2144,14 @@
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>1 runs on the P&amp;ID — metres not on the drawing</t>
+          <t>1 run on the P&amp;ID · 45 m off the drawing = 45 m</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>63mm tube pipe</t>
+          <t>101mm tube pipe</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2159,6 +2170,9 @@
           <t>ENGINEER</t>
         </is>
       </c>
+      <c r="G38" t="n">
+        <v>12</v>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
           <t>m</t>
@@ -2174,44 +2188,41 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>1 runs on the P&amp;ID — metres not on the drawing</t>
+          <t>1 run on the P&amp;ID · 12 m off the drawing = 12 m</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>76mm 304 press pipe</t>
+          <t>63mm tube pipe</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>M-PFS</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>PT-76</t>
-        </is>
-      </c>
+          <t>M-P</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" s="10" t="inlineStr">
         <is>
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F39" s="15" t="inlineStr">
-        <is>
-          <t>PRICE LIST</t>
-        </is>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>ENGINEER</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>12</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="I39" s="16" t="n">
-        <v>53.1</v>
-      </c>
+      <c r="I39" s="4" t="n"/>
       <c r="J39" s="17" t="n">
         <v>0.15</v>
       </c>
@@ -2221,14 +2232,14 @@
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>1 runs on the P&amp;ID — metres not on the drawing</t>
+          <t>1 run on the P&amp;ID · 12 m off the drawing = 12 m</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>54mm 304 press pipe</t>
+          <t>76mm 304 press pipe</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2238,7 +2249,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>PT-54</t>
+          <t>PT-76</t>
         </is>
       </c>
       <c r="E40" s="10" t="inlineStr">
@@ -2251,13 +2262,16 @@
           <t>PRICE LIST</t>
         </is>
       </c>
+      <c r="G40" t="n">
+        <v>10</v>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
       <c r="I40" s="16" t="n">
-        <v>17.4</v>
+        <v>53.1</v>
       </c>
       <c r="J40" s="17" t="n">
         <v>0.15</v>
@@ -2268,183 +2282,192 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>1 runs on the P&amp;ID — metres not on the drawing</t>
+          <t>1 run on the P&amp;ID · 10 m off the drawing = 10 m</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="19" t="inlineStr">
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>54mm 304 press pipe</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>M-PFS</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>PT-54</t>
+        </is>
+      </c>
+      <c r="E41" s="10" t="inlineStr">
+        <is>
+          <t>Bought in</t>
+        </is>
+      </c>
+      <c r="F41" s="15" t="inlineStr">
+        <is>
+          <t>PRICE LIST</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>10</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="I41" s="16" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="J41" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K41" s="4">
+        <f>IFERROR($G41*$I41,"")</f>
+        <v/>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>1 run on the P&amp;ID · 10 m off the drawing = 10 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="19" t="inlineStr">
         <is>
           <t>Pipe insulation</t>
         </is>
       </c>
-      <c r="C41" s="10" t="inlineStr">
+      <c r="C42" s="10" t="inlineStr">
         <is>
           <t>M-INS</t>
         </is>
       </c>
-      <c r="D41" s="10" t="inlineStr"/>
-      <c r="E41" s="10" t="inlineStr">
+      <c r="D42" s="10" t="inlineStr"/>
+      <c r="E42" s="10" t="inlineStr">
         <is>
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F41" s="10" t="inlineStr">
+      <c r="F42" s="10" t="inlineStr">
         <is>
           <t>RATE</t>
         </is>
       </c>
-      <c r="G41" s="10" t="n"/>
-      <c r="H41" s="10" t="inlineStr">
+      <c r="G42" s="10" t="n">
+        <v>243</v>
+      </c>
+      <c r="H42" s="10" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="I41" s="20" t="n"/>
-      <c r="J41" s="21" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K41" s="20">
-        <f>IFERROR($G41*$I41,"")</f>
-        <v/>
-      </c>
-      <c r="L41" s="22" t="inlineStr">
-        <is>
-          <t>rate card by diameter</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="B42" s="14" t="inlineStr">
+      <c r="I42" s="20" t="n"/>
+      <c r="J42" s="21" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K42" s="20">
+        <f>IFERROR($G42*$I42,"")</f>
+        <v/>
+      </c>
+      <c r="L42" s="22" t="inlineStr">
+        <is>
+          <t>17 insulated runs · 243 m off the drawing (drains excluded)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="14" t="inlineStr">
         <is>
           <t>Freight and cartage</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>P-FRE</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" s="10" t="inlineStr">
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" s="10" t="inlineStr">
         <is>
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>lot</t>
         </is>
       </c>
-      <c r="I42" s="4" t="n"/>
-      <c r="J42" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K42" s="4">
-        <f>IFERROR($G42*$I42,"")</f>
-        <v/>
-      </c>
-      <c r="L42" s="2" t="inlineStr">
+      <c r="I43" s="4" t="n"/>
+      <c r="J43" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K43" s="4">
+        <f>IFERROR($G43*$I43,"")</f>
+        <v/>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
         <is>
           <t>carried on past jobs</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="3" t="n"/>
-      <c r="B43" s="3" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="3" t="n"/>
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>Section 7.6 total</t>
         </is>
       </c>
-      <c r="C43" s="3" t="n"/>
-      <c r="D43" s="3" t="n"/>
-      <c r="E43" s="3" t="n"/>
-      <c r="F43" s="3" t="n"/>
-      <c r="G43" s="3" t="n"/>
-      <c r="H43" s="3" t="n"/>
-      <c r="I43" s="3" t="n"/>
-      <c r="J43" s="3" t="n"/>
-      <c r="K43" s="18">
-        <f>SUM(K24:K42)</f>
-        <v/>
-      </c>
-      <c r="L43" s="3" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="7" t="inlineStr">
+      <c r="C44" s="3" t="n"/>
+      <c r="D44" s="3" t="n"/>
+      <c r="E44" s="3" t="n"/>
+      <c r="F44" s="3" t="n"/>
+      <c r="G44" s="3" t="n"/>
+      <c r="H44" s="3" t="n"/>
+      <c r="I44" s="3" t="n"/>
+      <c r="J44" s="3" t="n"/>
+      <c r="K44" s="18">
+        <f>SUM(K24:K43)</f>
+        <v/>
+      </c>
+      <c r="L44" s="3" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
         <is>
           <t>7.7</t>
         </is>
       </c>
-      <c r="B44" s="7" t="inlineStr">
+      <c r="B45" s="7" t="inlineStr">
         <is>
           <t>Installation labour, supervision and consumables</t>
         </is>
       </c>
-      <c r="C44" s="7" t="n"/>
-      <c r="D44" s="7" t="n"/>
-      <c r="E44" s="7" t="n"/>
-      <c r="F44" s="7" t="n"/>
-      <c r="G44" s="7" t="n"/>
-      <c r="H44" s="7" t="n"/>
-      <c r="I44" s="7" t="n"/>
-      <c r="J44" s="7" t="n"/>
-      <c r="K44" s="7" t="n"/>
-      <c r="L44" s="7" t="n"/>
-    </row>
-    <row r="45">
-      <c r="B45" s="14" t="inlineStr">
-        <is>
-          <t>Set out and rig plant</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>L-SERVIN</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" s="15" t="inlineStr">
-        <is>
-          <t>In-house</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>ENGINEER</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>hr</t>
-        </is>
-      </c>
-      <c r="I45" s="4" t="n">
-        <v>105</v>
-      </c>
-      <c r="J45" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K45" s="4">
-        <f>IFERROR($G45*$I45,"")</f>
-        <v/>
-      </c>
-      <c r="L45" s="2" t="inlineStr">
-        <is>
-          <t>crew × days</t>
-        </is>
-      </c>
+      <c r="C45" s="7" t="n"/>
+      <c r="D45" s="7" t="n"/>
+      <c r="E45" s="7" t="n"/>
+      <c r="F45" s="7" t="n"/>
+      <c r="G45" s="7" t="n"/>
+      <c r="H45" s="7" t="n"/>
+      <c r="I45" s="7" t="n"/>
+      <c r="J45" s="7" t="n"/>
+      <c r="K45" s="7" t="n"/>
+      <c r="L45" s="7" t="n"/>
     </row>
     <row r="46">
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>Pipe compressor pack</t>
+          <t>Set out and rig plant</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2487,7 +2510,7 @@
     <row r="47">
       <c r="B47" s="14" t="inlineStr">
         <is>
-          <t>Pipe chiller and glycol circuit</t>
+          <t>Pipe compressor pack</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2530,7 +2553,7 @@
     <row r="48">
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>Hang and pipe unit coolers</t>
+          <t>Pipe chiller and glycol circuit</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2573,7 +2596,7 @@
     <row r="49">
       <c r="B49" s="14" t="inlineStr">
         <is>
-          <t>Pressure test</t>
+          <t>Hang and pipe unit coolers</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2616,7 +2639,7 @@
     <row r="50">
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t>Insulate</t>
+          <t>Pressure test</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2659,7 +2682,7 @@
     <row r="51">
       <c r="B51" s="14" t="inlineStr">
         <is>
-          <t>Glycol fill and flush</t>
+          <t>Insulate</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2702,7 +2725,7 @@
     <row r="52">
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>Changeover weekend</t>
+          <t>Glycol fill and flush</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2745,7 +2768,7 @@
     <row r="53">
       <c r="B53" s="14" t="inlineStr">
         <is>
-          <t>Supervision</t>
+          <t>Changeover weekend</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2788,18 +2811,18 @@
     <row r="54">
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>Crane and access hire</t>
+          <t>Supervision</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>P-HIRE</t>
+          <t>L-SERVIN</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
-      <c r="E54" s="10" t="inlineStr">
-        <is>
-          <t>Bought in</t>
+      <c r="E54" s="15" t="inlineStr">
+        <is>
+          <t>In-house</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2809,10 +2832,12 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>lot</t>
-        </is>
-      </c>
-      <c r="I54" s="4" t="n"/>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="I54" s="4" t="n">
+        <v>105</v>
+      </c>
       <c r="J54" s="17" t="n">
         <v>0.15</v>
       </c>
@@ -2822,19 +2847,19 @@
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>carried on past jobs</t>
+          <t>crew × days</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="B55" s="14" t="inlineStr">
         <is>
-          <t>Travel and accommodation</t>
+          <t>Crane and access hire</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>D-TRAV</t>
+          <t>P-HIRE</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -2870,12 +2895,12 @@
     <row r="56">
       <c r="B56" s="14" t="inlineStr">
         <is>
-          <t>Site setup and safety</t>
+          <t>Travel and accommodation</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>P-SS</t>
+          <t>D-TRAV</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -2909,148 +2934,145 @@
       </c>
     </row>
     <row r="57">
-      <c r="B57" s="15" t="inlineStr">
+      <c r="B57" s="14" t="inlineStr">
+        <is>
+          <t>Site setup and safety</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>P-SS</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" s="10" t="inlineStr">
+        <is>
+          <t>Bought in</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>ENGINEER</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="I57" s="4" t="n"/>
+      <c r="J57" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K57" s="4">
+        <f>IFERROR($G57*$I57,"")</f>
+        <v/>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>carried on past jobs</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="15" t="inlineStr">
         <is>
           <t>Site welding and fit-up</t>
         </is>
       </c>
-      <c r="C57" s="15" t="inlineStr">
+      <c r="C58" s="15" t="inlineStr">
         <is>
           <t>L-SERVIN</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" s="15" t="inlineStr">
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" s="15" t="inlineStr">
         <is>
           <t>In-house</t>
         </is>
       </c>
-      <c r="F57" s="15" t="inlineStr">
+      <c r="F58" s="15" t="inlineStr">
         <is>
           <t>TAKE-OFF</t>
         </is>
       </c>
-      <c r="G57" s="23">
-        <f>'Take-off'!F20</f>
-        <v/>
-      </c>
-      <c r="H57" s="15" t="inlineStr">
+      <c r="G58" s="23">
+        <f>'Take-off'!F16</f>
+        <v/>
+      </c>
+      <c r="H58" s="15" t="inlineStr">
         <is>
           <t>hr</t>
         </is>
       </c>
-      <c r="I57" s="16" t="n">
+      <c r="I58" s="16" t="n">
         <v>110</v>
       </c>
-      <c r="J57" s="24" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K57" s="16">
-        <f>IFERROR($G57*$I57,"")</f>
-        <v/>
-      </c>
-      <c r="L57" s="25" t="inlineStr">
+      <c r="J58" s="24" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K58" s="16">
+        <f>IFERROR($G58*$I58,"")</f>
+        <v/>
+      </c>
+      <c r="L58" s="25" t="inlineStr">
         <is>
           <t>hours from the Take-off, priced off the Welding hours matrix</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="3" t="n"/>
-      <c r="B58" s="3" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="3" t="n"/>
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>Section 7.7 total</t>
         </is>
       </c>
-      <c r="C58" s="3" t="n"/>
-      <c r="D58" s="3" t="n"/>
-      <c r="E58" s="3" t="n"/>
-      <c r="F58" s="3" t="n"/>
-      <c r="G58" s="3" t="n"/>
-      <c r="H58" s="3" t="n"/>
-      <c r="I58" s="3" t="n"/>
-      <c r="J58" s="3" t="n"/>
-      <c r="K58" s="18">
-        <f>SUM(K45:K57)</f>
-        <v/>
-      </c>
-      <c r="L58" s="3" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="7" t="inlineStr">
+      <c r="C59" s="3" t="n"/>
+      <c r="D59" s="3" t="n"/>
+      <c r="E59" s="3" t="n"/>
+      <c r="F59" s="3" t="n"/>
+      <c r="G59" s="3" t="n"/>
+      <c r="H59" s="3" t="n"/>
+      <c r="I59" s="3" t="n"/>
+      <c r="J59" s="3" t="n"/>
+      <c r="K59" s="18">
+        <f>SUM(K46:K58)</f>
+        <v/>
+      </c>
+      <c r="L59" s="3" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="7" t="inlineStr">
         <is>
           <t>7.8</t>
         </is>
       </c>
-      <c r="B59" s="7" t="inlineStr">
+      <c r="B60" s="7" t="inlineStr">
         <is>
           <t>Electrical power, control wiring and SCADA</t>
         </is>
       </c>
-      <c r="C59" s="7" t="n"/>
-      <c r="D59" s="7" t="n"/>
-      <c r="E59" s="7" t="n"/>
-      <c r="F59" s="7" t="n"/>
-      <c r="G59" s="7" t="n"/>
-      <c r="H59" s="7" t="n"/>
-      <c r="I59" s="7" t="n"/>
-      <c r="J59" s="7" t="n"/>
-      <c r="K59" s="7" t="n"/>
-      <c r="L59" s="7" t="n"/>
-    </row>
-    <row r="60">
-      <c r="B60" s="8" t="inlineStr">
-        <is>
-          <t>Power and control wiring</t>
-        </is>
-      </c>
-      <c r="C60" s="9" t="inlineStr">
-        <is>
-          <t>ES-INST</t>
-        </is>
-      </c>
-      <c r="D60" s="9" t="inlineStr"/>
-      <c r="E60" s="9" t="inlineStr">
-        <is>
-          <t>Subcontract</t>
-        </is>
-      </c>
-      <c r="F60" s="9" t="inlineStr">
-        <is>
-          <t>RFQ</t>
-        </is>
-      </c>
-      <c r="G60" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="H60" s="9" t="inlineStr">
-        <is>
-          <t>lot</t>
-        </is>
-      </c>
-      <c r="I60" s="11" t="n"/>
-      <c r="J60" s="12" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K60" s="11">
-        <f>IFERROR($G60*$I60,"")</f>
-        <v/>
-      </c>
-      <c r="L60" s="13" t="inlineStr">
-        <is>
-          <t>from the maximum demand schedule</t>
-        </is>
-      </c>
+      <c r="C60" s="7" t="n"/>
+      <c r="D60" s="7" t="n"/>
+      <c r="E60" s="7" t="n"/>
+      <c r="F60" s="7" t="n"/>
+      <c r="G60" s="7" t="n"/>
+      <c r="H60" s="7" t="n"/>
+      <c r="I60" s="7" t="n"/>
+      <c r="J60" s="7" t="n"/>
+      <c r="K60" s="7" t="n"/>
+      <c r="L60" s="7" t="n"/>
     </row>
     <row r="61">
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>SCADA integration — Ignition</t>
+          <t>Power and control wiring</t>
         </is>
       </c>
       <c r="C61" s="9" t="inlineStr">
         <is>
-          <t>ES-AU</t>
+          <t>ES-INST</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr"/>
@@ -3082,100 +3104,101 @@
       </c>
       <c r="L61" s="13" t="inlineStr">
         <is>
+          <t>from the maximum demand schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="8" t="inlineStr">
+        <is>
+          <t>SCADA integration — Ignition</t>
+        </is>
+      </c>
+      <c r="C62" s="9" t="inlineStr">
+        <is>
+          <t>ES-AU</t>
+        </is>
+      </c>
+      <c r="D62" s="9" t="inlineStr"/>
+      <c r="E62" s="9" t="inlineStr">
+        <is>
+          <t>Subcontract</t>
+        </is>
+      </c>
+      <c r="F62" s="9" t="inlineStr">
+        <is>
+          <t>RFQ</t>
+        </is>
+      </c>
+      <c r="G62" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H62" s="9" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="I62" s="11" t="n"/>
+      <c r="J62" s="12" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K62" s="11">
+        <f>IFERROR($G62*$I62,"")</f>
+        <v/>
+      </c>
+      <c r="L62" s="13" t="inlineStr">
+        <is>
           <t>electrical contractor</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="3" t="n"/>
-      <c r="B62" s="3" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="3" t="n"/>
+      <c r="B63" s="3" t="inlineStr">
         <is>
           <t>Section 7.8 total</t>
         </is>
       </c>
-      <c r="C62" s="3" t="n"/>
-      <c r="D62" s="3" t="n"/>
-      <c r="E62" s="3" t="n"/>
-      <c r="F62" s="3" t="n"/>
-      <c r="G62" s="3" t="n"/>
-      <c r="H62" s="3" t="n"/>
-      <c r="I62" s="3" t="n"/>
-      <c r="J62" s="3" t="n"/>
-      <c r="K62" s="18">
-        <f>SUM(K60:K61)</f>
-        <v/>
-      </c>
-      <c r="L62" s="3" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="7" t="inlineStr">
+      <c r="C63" s="3" t="n"/>
+      <c r="D63" s="3" t="n"/>
+      <c r="E63" s="3" t="n"/>
+      <c r="F63" s="3" t="n"/>
+      <c r="G63" s="3" t="n"/>
+      <c r="H63" s="3" t="n"/>
+      <c r="I63" s="3" t="n"/>
+      <c r="J63" s="3" t="n"/>
+      <c r="K63" s="18">
+        <f>SUM(K61:K62)</f>
+        <v/>
+      </c>
+      <c r="L63" s="3" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="inlineStr">
         <is>
           <t>7.9</t>
         </is>
       </c>
-      <c r="B63" s="7" t="inlineStr">
+      <c r="B64" s="7" t="inlineStr">
         <is>
           <t>As-built documentation, training, O&amp;M</t>
         </is>
       </c>
-      <c r="C63" s="7" t="n"/>
-      <c r="D63" s="7" t="n"/>
-      <c r="E63" s="7" t="n"/>
-      <c r="F63" s="7" t="n"/>
-      <c r="G63" s="7" t="n"/>
-      <c r="H63" s="7" t="n"/>
-      <c r="I63" s="7" t="n"/>
-      <c r="J63" s="7" t="n"/>
-      <c r="K63" s="7" t="n"/>
-      <c r="L63" s="7" t="n"/>
-    </row>
-    <row r="64">
-      <c r="B64" s="14" t="inlineStr">
-        <is>
-          <t>As-built drawings</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>L-DWG</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" s="15" t="inlineStr">
-        <is>
-          <t>In-house</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>ENGINEER</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>hr</t>
-        </is>
-      </c>
-      <c r="I64" s="4" t="n">
-        <v>140</v>
-      </c>
-      <c r="J64" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K64" s="4">
-        <f>IFERROR($G64*$I64,"")</f>
-        <v/>
-      </c>
-      <c r="L64" s="2" t="inlineStr">
-        <is>
-          <t>hours to be entered</t>
-        </is>
-      </c>
+      <c r="C64" s="7" t="n"/>
+      <c r="D64" s="7" t="n"/>
+      <c r="E64" s="7" t="n"/>
+      <c r="F64" s="7" t="n"/>
+      <c r="G64" s="7" t="n"/>
+      <c r="H64" s="7" t="n"/>
+      <c r="I64" s="7" t="n"/>
+      <c r="J64" s="7" t="n"/>
+      <c r="K64" s="7" t="n"/>
+      <c r="L64" s="7" t="n"/>
     </row>
     <row r="65">
       <c r="B65" s="14" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>As-built drawings</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3218,7 +3241,7 @@
     <row r="66">
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t>O&amp;M manuals</t>
+          <t>Training</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3261,12 +3284,12 @@
     <row r="67">
       <c r="B67" s="14" t="inlineStr">
         <is>
-          <t>Producer statements</t>
+          <t>O&amp;M manuals</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>L-DV</t>
+          <t>L-DWG</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -3304,18 +3327,18 @@
     <row r="68">
       <c r="B68" s="14" t="inlineStr">
         <is>
-          <t>Compliance and inspection</t>
+          <t>Producer statements</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>P-RCOMP</t>
+          <t>L-DV</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
-      <c r="E68" s="10" t="inlineStr">
-        <is>
-          <t>Bought in</t>
+      <c r="E68" s="15" t="inlineStr">
+        <is>
+          <t>In-house</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3325,10 +3348,12 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>lot</t>
-        </is>
-      </c>
-      <c r="I68" s="4" t="n"/>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="I68" s="4" t="n">
+        <v>140</v>
+      </c>
       <c r="J68" s="17" t="n">
         <v>0.15</v>
       </c>
@@ -3338,111 +3363,109 @@
       </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
+          <t>hours to be entered</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="14" t="inlineStr">
+        <is>
+          <t>Compliance and inspection</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>P-RCOMP</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" s="10" t="inlineStr">
+        <is>
+          <t>Bought in</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>ENGINEER</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="I69" s="4" t="n"/>
+      <c r="J69" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K69" s="4">
+        <f>IFERROR($G69*$I69,"")</f>
+        <v/>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
           <t>carried on past jobs</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="3" t="n"/>
-      <c r="B69" s="3" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="3" t="n"/>
+      <c r="B70" s="3" t="inlineStr">
         <is>
           <t>Section 7.9 total</t>
         </is>
       </c>
-      <c r="C69" s="3" t="n"/>
-      <c r="D69" s="3" t="n"/>
-      <c r="E69" s="3" t="n"/>
-      <c r="F69" s="3" t="n"/>
-      <c r="G69" s="3" t="n"/>
-      <c r="H69" s="3" t="n"/>
-      <c r="I69" s="3" t="n"/>
-      <c r="J69" s="3" t="n"/>
-      <c r="K69" s="18">
-        <f>SUM(K64:K68)</f>
-        <v/>
-      </c>
-      <c r="L69" s="3" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="7" t="inlineStr">
+      <c r="C70" s="3" t="n"/>
+      <c r="D70" s="3" t="n"/>
+      <c r="E70" s="3" t="n"/>
+      <c r="F70" s="3" t="n"/>
+      <c r="G70" s="3" t="n"/>
+      <c r="H70" s="3" t="n"/>
+      <c r="I70" s="3" t="n"/>
+      <c r="J70" s="3" t="n"/>
+      <c r="K70" s="18">
+        <f>SUM(K65:K69)</f>
+        <v/>
+      </c>
+      <c r="L70" s="3" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="7" t="inlineStr">
         <is>
           <t>7.10</t>
         </is>
       </c>
-      <c r="B70" s="7" t="inlineStr">
+      <c r="B71" s="7" t="inlineStr">
         <is>
           <t>Commissioning, glycol charge and spares</t>
         </is>
       </c>
-      <c r="C70" s="7" t="n"/>
-      <c r="D70" s="7" t="n"/>
-      <c r="E70" s="7" t="n"/>
-      <c r="F70" s="7" t="n"/>
-      <c r="G70" s="7" t="n"/>
-      <c r="H70" s="7" t="n"/>
-      <c r="I70" s="7" t="n"/>
-      <c r="J70" s="7" t="n"/>
-      <c r="K70" s="7" t="n"/>
-      <c r="L70" s="7" t="n"/>
-    </row>
-    <row r="71">
-      <c r="B71" s="14" t="inlineStr">
-        <is>
-          <t>Commissioning and pulldown demonstration</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>L-COM</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" s="15" t="inlineStr">
-        <is>
-          <t>In-house</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>ENGINEER</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>hr</t>
-        </is>
-      </c>
-      <c r="I71" s="4" t="n">
-        <v>105</v>
-      </c>
-      <c r="J71" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K71" s="4">
-        <f>IFERROR($G71*$I71,"")</f>
-        <v/>
-      </c>
-      <c r="L71" s="2" t="inlineStr">
-        <is>
-          <t>to be entered</t>
-        </is>
-      </c>
+      <c r="C71" s="7" t="n"/>
+      <c r="D71" s="7" t="n"/>
+      <c r="E71" s="7" t="n"/>
+      <c r="F71" s="7" t="n"/>
+      <c r="G71" s="7" t="n"/>
+      <c r="H71" s="7" t="n"/>
+      <c r="I71" s="7" t="n"/>
+      <c r="J71" s="7" t="n"/>
+      <c r="K71" s="7" t="n"/>
+      <c r="L71" s="7" t="n"/>
     </row>
     <row r="72">
       <c r="B72" s="14" t="inlineStr">
         <is>
-          <t>Glycol charge — MPG 35%</t>
+          <t>Commissioning and pulldown demonstration</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>R-GLY</t>
+          <t>L-COM</t>
         </is>
       </c>
       <c r="D72" t="inlineStr"/>
-      <c r="E72" s="10" t="inlineStr">
-        <is>
-          <t>Bought in</t>
+      <c r="E72" s="15" t="inlineStr">
+        <is>
+          <t>In-house</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3452,10 +3475,12 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I72" s="4" t="n"/>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="I72" s="4" t="n">
+        <v>105</v>
+      </c>
       <c r="J72" s="17" t="n">
         <v>0.15</v>
       </c>
@@ -3472,12 +3497,12 @@
     <row r="73">
       <c r="B73" s="14" t="inlineStr">
         <is>
-          <t>Spare parts</t>
+          <t>Glycol charge — MPG 35%</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>M-GEN</t>
+          <t>R-GLY</t>
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
@@ -3493,7 +3518,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>ea</t>
+          <t>L</t>
         </is>
       </c>
       <c r="I73" s="4" t="n"/>
@@ -3511,101 +3536,98 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="3" t="n"/>
-      <c r="B74" s="3" t="inlineStr">
+      <c r="B74" s="14" t="inlineStr">
+        <is>
+          <t>Spare parts</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>M-GEN</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" s="10" t="inlineStr">
+        <is>
+          <t>Bought in</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>ENGINEER</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I74" s="4" t="n"/>
+      <c r="J74" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K74" s="4">
+        <f>IFERROR($G74*$I74,"")</f>
+        <v/>
+      </c>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>to be entered</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="n"/>
+      <c r="B75" s="3" t="inlineStr">
         <is>
           <t>Section 7.10 total</t>
         </is>
       </c>
-      <c r="C74" s="3" t="n"/>
-      <c r="D74" s="3" t="n"/>
-      <c r="E74" s="3" t="n"/>
-      <c r="F74" s="3" t="n"/>
-      <c r="G74" s="3" t="n"/>
-      <c r="H74" s="3" t="n"/>
-      <c r="I74" s="3" t="n"/>
-      <c r="J74" s="3" t="n"/>
-      <c r="K74" s="18">
-        <f>SUM(K71:K73)</f>
-        <v/>
-      </c>
-      <c r="L74" s="3" t="n"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="7" t="inlineStr">
+      <c r="C75" s="3" t="n"/>
+      <c r="D75" s="3" t="n"/>
+      <c r="E75" s="3" t="n"/>
+      <c r="F75" s="3" t="n"/>
+      <c r="G75" s="3" t="n"/>
+      <c r="H75" s="3" t="n"/>
+      <c r="I75" s="3" t="n"/>
+      <c r="J75" s="3" t="n"/>
+      <c r="K75" s="18">
+        <f>SUM(K72:K74)</f>
+        <v/>
+      </c>
+      <c r="L75" s="3" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="7" t="inlineStr">
         <is>
           <t>7.11</t>
         </is>
       </c>
-      <c r="B75" s="7" t="inlineStr">
+      <c r="B76" s="7" t="inlineStr">
         <is>
           <t>Twelve months defects liability and routine maintenance</t>
         </is>
       </c>
-      <c r="C75" s="7" t="n"/>
-      <c r="D75" s="7" t="n"/>
-      <c r="E75" s="7" t="n"/>
-      <c r="F75" s="7" t="n"/>
-      <c r="G75" s="7" t="n"/>
-      <c r="H75" s="7" t="n"/>
-      <c r="I75" s="7" t="n"/>
-      <c r="J75" s="7" t="n"/>
-      <c r="K75" s="7" t="n"/>
-      <c r="L75" s="7" t="n"/>
-    </row>
-    <row r="76">
-      <c r="B76" s="14" t="inlineStr">
-        <is>
-          <t>Routine maintenance, 12 months</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>D-MAINT</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr"/>
-      <c r="E76" s="10" t="inlineStr">
-        <is>
-          <t>Bought in</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>ENGINEER</t>
-        </is>
-      </c>
-      <c r="G76" t="n">
-        <v>4</v>
-      </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>visit</t>
-        </is>
-      </c>
-      <c r="I76" s="4" t="n"/>
-      <c r="J76" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K76" s="4">
-        <f>IFERROR($G76*$I76,"")</f>
-        <v/>
-      </c>
-      <c r="L76" s="2" t="inlineStr">
-        <is>
-          <t>rate to be entered</t>
-        </is>
-      </c>
+      <c r="C76" s="7" t="n"/>
+      <c r="D76" s="7" t="n"/>
+      <c r="E76" s="7" t="n"/>
+      <c r="F76" s="7" t="n"/>
+      <c r="G76" s="7" t="n"/>
+      <c r="H76" s="7" t="n"/>
+      <c r="I76" s="7" t="n"/>
+      <c r="J76" s="7" t="n"/>
+      <c r="K76" s="7" t="n"/>
+      <c r="L76" s="7" t="n"/>
     </row>
     <row r="77">
       <c r="B77" s="14" t="inlineStr">
         <is>
-          <t>Contingency</t>
+          <t>Routine maintenance, 12 months</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>D-CONT</t>
+          <t>D-MAINT</t>
         </is>
       </c>
       <c r="D77" t="inlineStr"/>
@@ -3619,9 +3641,12 @@
           <t>ENGINEER</t>
         </is>
       </c>
+      <c r="G77" t="n">
+        <v>4</v>
+      </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>visit</t>
         </is>
       </c>
       <c r="I77" s="4" t="n"/>
@@ -3634,55 +3659,96 @@
       </c>
       <c r="L77" s="2" t="inlineStr">
         <is>
+          <t>rate to be entered</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="14" t="inlineStr">
+        <is>
+          <t>Contingency</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>D-CONT</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" s="10" t="inlineStr">
+        <is>
+          <t>Bought in</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>ENGINEER</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="I78" s="4" t="n"/>
+      <c r="J78" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K78" s="4">
+        <f>IFERROR($G78*$I78,"")</f>
+        <v/>
+      </c>
+      <c r="L78" s="2" t="inlineStr">
+        <is>
           <t>carried on past jobs</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="3" t="n"/>
-      <c r="B78" s="3" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="3" t="n"/>
+      <c r="B79" s="3" t="inlineStr">
         <is>
           <t>Section 7.11 total</t>
         </is>
       </c>
-      <c r="C78" s="3" t="n"/>
-      <c r="D78" s="3" t="n"/>
-      <c r="E78" s="3" t="n"/>
-      <c r="F78" s="3" t="n"/>
-      <c r="G78" s="3" t="n"/>
-      <c r="H78" s="3" t="n"/>
-      <c r="I78" s="3" t="n"/>
-      <c r="J78" s="3" t="n"/>
-      <c r="K78" s="18">
-        <f>SUM(K76:K77)</f>
-        <v/>
-      </c>
-      <c r="L78" s="3" t="n"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="3" t="n"/>
-      <c r="B80" s="3" t="inlineStr">
+      <c r="C79" s="3" t="n"/>
+      <c r="D79" s="3" t="n"/>
+      <c r="E79" s="3" t="n"/>
+      <c r="F79" s="3" t="n"/>
+      <c r="G79" s="3" t="n"/>
+      <c r="H79" s="3" t="n"/>
+      <c r="I79" s="3" t="n"/>
+      <c r="J79" s="3" t="n"/>
+      <c r="K79" s="18">
+        <f>SUM(K77:K78)</f>
+        <v/>
+      </c>
+      <c r="L79" s="3" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="n"/>
+      <c r="B81" s="3" t="inlineStr">
         <is>
           <t>TOTAL COST</t>
         </is>
       </c>
-      <c r="C80" s="3" t="n"/>
-      <c r="D80" s="3" t="n"/>
-      <c r="E80" s="3" t="n"/>
-      <c r="F80" s="3" t="n"/>
-      <c r="G80" s="3" t="n"/>
-      <c r="H80" s="3" t="n"/>
-      <c r="I80" s="3" t="n"/>
-      <c r="J80" s="3" t="n"/>
-      <c r="K80" s="18">
-        <f>K9+K12+K15+K19+K22+K43+K58+K62+K69+K74+K78</f>
-        <v/>
-      </c>
-      <c r="L80" s="3" t="n"/>
+      <c r="C81" s="3" t="n"/>
+      <c r="D81" s="3" t="n"/>
+      <c r="E81" s="3" t="n"/>
+      <c r="F81" s="3" t="n"/>
+      <c r="G81" s="3" t="n"/>
+      <c r="H81" s="3" t="n"/>
+      <c r="I81" s="3" t="n"/>
+      <c r="J81" s="3" t="n"/>
+      <c r="K81" s="18">
+        <f>K9+K12+K15+K19+K22+K44+K59+K63+K70+K75+K79</f>
+        <v/>
+      </c>
+      <c r="L81" s="3" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="E45 E46 E47 E48 E49 E50 E51 E52 E53 E57 E60 E61 E64 E65 E66 E67 E71" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E46 E47 E48 E49 E50 E51 E52 E53 E54 E58 E61 E62 E65 E66 E67 E68 E72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"In-house,Subcontract"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3860,7 +3926,7 @@
         </is>
       </c>
       <c r="C7" s="4">
-        <f>Costing!K43</f>
+        <f>Costing!K44</f>
         <v/>
       </c>
       <c r="D7" s="17" t="n">
@@ -3883,7 +3949,7 @@
         </is>
       </c>
       <c r="C8" s="4">
-        <f>Costing!K58</f>
+        <f>Costing!K59</f>
         <v/>
       </c>
       <c r="D8" s="17" t="n">
@@ -3906,7 +3972,7 @@
         </is>
       </c>
       <c r="C9" s="4">
-        <f>Costing!K62</f>
+        <f>Costing!K63</f>
         <v/>
       </c>
       <c r="D9" s="17" t="n">
@@ -3929,7 +3995,7 @@
         </is>
       </c>
       <c r="C10" s="4">
-        <f>Costing!K69</f>
+        <f>Costing!K70</f>
         <v/>
       </c>
       <c r="D10" s="17" t="n">
@@ -3952,7 +4018,7 @@
         </is>
       </c>
       <c r="C11" s="4">
-        <f>Costing!K74</f>
+        <f>Costing!K75</f>
         <v/>
       </c>
       <c r="D11" s="17" t="n">
@@ -3975,7 +4041,7 @@
         </is>
       </c>
       <c r="C12" s="4">
-        <f>Costing!K78</f>
+        <f>Costing!K79</f>
         <v/>
       </c>
       <c r="D12" s="17" t="n">
@@ -4625,7 +4691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4804,7 +4870,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -4819,7 +4885,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -4875,8 +4941,11 @@
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
-          <t>100NB pipe</t>
-        </is>
+          <t>80NB pipe</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>98</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -4887,8 +4956,11 @@
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
-          <t>80NB pipe</t>
-        </is>
+          <t>100NB pipe</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>8</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -4899,8 +4971,11 @@
     <row r="18">
       <c r="B18" t="inlineStr">
         <is>
-          <t>101mm tube pipe</t>
-        </is>
+          <t>50NB pipe</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>45</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -4911,8 +4986,11 @@
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
-          <t>63mm tube pipe</t>
-        </is>
+          <t>101mm tube pipe</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>12</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -4923,8 +5001,11 @@
     <row r="20">
       <c r="B20" t="inlineStr">
         <is>
-          <t>Pipe insulation</t>
-        </is>
+          <t>63mm tube pipe</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>12</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -4935,82 +5016,100 @@
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
+          <t>Pipe insulation</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>243</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
           <t>Spare parts</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>Pipe insulation</t>
         </is>
       </c>
-      <c r="B22" s="7" t="n"/>
-      <c r="C22" s="7" t="n"/>
-      <c r="D22" s="7" t="n"/>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="B23" s="7" t="n"/>
+      <c r="C23" s="7" t="n"/>
+      <c r="D23" s="7" t="n"/>
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>insulation subcontractor — request a schedule of rates, $/m by diameter</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" t="inlineStr">
+    <row r="24">
+      <c r="B24" t="inlineStr">
         <is>
           <t>Pipe insulation</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="C24" t="n">
+        <v>243</v>
+      </c>
+      <c r="D24" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>Electrical power, control wiring and SCADA</t>
         </is>
       </c>
-      <c r="B24" s="7" t="n"/>
-      <c r="C24" s="7" t="n"/>
-      <c r="D24" s="7" t="n"/>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="B25" s="7" t="n"/>
+      <c r="C25" s="7" t="n"/>
+      <c r="D25" s="7" t="n"/>
+      <c r="E25" s="7" t="inlineStr">
         <is>
           <t>electrical contractor — attach the Electrical tab</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Power and control wiring</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>lot</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" t="inlineStr">
         <is>
-          <t>SCADA integration — Ignition</t>
+          <t>Power and control wiring</t>
         </is>
       </c>
       <c r="C26" t="n">
         <v>1</v>
       </c>
       <c r="D26" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>SCADA integration — Ignition</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" t="inlineStr">
         <is>
           <t>lot</t>
         </is>
@@ -5027,7 +5126,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5093,7 +5192,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E2" s="26">
         <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B2,'Welding hours'!$C$3:$C$14,0),MATCH($C2,'Welding hours'!$D$2:$O$2,0)),0)</f>
@@ -5159,7 +5258,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E4" s="26">
         <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B4,'Welding hours'!$C$3:$C$14,0),MATCH($C4,'Welding hours'!$D$2:$O$2,0)),0)</f>
@@ -5407,237 +5506,119 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>42mm 304 press</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>1 1/2"</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>Straight</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="27">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>80NB</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>3"</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Buttweld</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>17</v>
+      </c>
+      <c r="E12" s="26">
         <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B12,'Welding hours'!$C$3:$C$14,0),MATCH($C12,'Welding hours'!$D$2:$O$2,0)),0)</f>
         <v/>
       </c>
-      <c r="F12" s="27">
+      <c r="F12" s="26">
         <f>D12*E12</f>
         <v/>
       </c>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>one weld per 6 m stick — enter the number of sticks</t>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>98 m off the drawing → 17 joints at one per 6 m stick</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>100NB</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>4"</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>Straight</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="27">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Buttweld</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" s="26">
         <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B13,'Welding hours'!$C$3:$C$14,0),MATCH($C13,'Welding hours'!$D$2:$O$2,0)),0)</f>
         <v/>
       </c>
-      <c r="F13" s="27">
+      <c r="F13" s="26">
         <f>D13*E13</f>
         <v/>
       </c>
-      <c r="G13" s="10" t="inlineStr">
-        <is>
-          <t>one weld per 6 m stick — enter the number of sticks</t>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>8 m off the drawing → 2 joints at one per 6 m stick</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>80NB</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>3"</t>
-        </is>
-      </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>Straight</t>
-        </is>
-      </c>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="27">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>50NB</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2"</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Buttweld</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>8</v>
+      </c>
+      <c r="E14" s="26">
         <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B14,'Welding hours'!$C$3:$C$14,0),MATCH($C14,'Welding hours'!$D$2:$O$2,0)),0)</f>
         <v/>
       </c>
-      <c r="F14" s="27">
+      <c r="F14" s="26">
         <f>D14*E14</f>
         <v/>
       </c>
-      <c r="G14" s="10" t="inlineStr">
-        <is>
-          <t>one weld per 6 m stick — enter the number of sticks</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>101mm tube</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>4"</t>
-        </is>
-      </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>Straight</t>
-        </is>
-      </c>
-      <c r="D15" s="10" t="n"/>
-      <c r="E15" s="27">
-        <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B15,'Welding hours'!$C$3:$C$14,0),MATCH($C15,'Welding hours'!$D$2:$O$2,0)),0)</f>
-        <v/>
-      </c>
-      <c r="F15" s="27">
-        <f>D15*E15</f>
-        <v/>
-      </c>
-      <c r="G15" s="10" t="inlineStr">
-        <is>
-          <t>one weld per 6 m stick — enter the number of sticks</t>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>45 m off the drawing → 8 joints at one per 6 m stick</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>63mm tube</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>2 1/2"</t>
-        </is>
-      </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>Straight</t>
-        </is>
-      </c>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="27">
-        <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B16,'Welding hours'!$C$3:$C$14,0),MATCH($C16,'Welding hours'!$D$2:$O$2,0)),0)</f>
-        <v/>
-      </c>
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL WELDING HOURS</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="3" t="n"/>
+      <c r="E16" s="3" t="n"/>
       <c r="F16" s="27">
-        <f>D16*E16</f>
-        <v/>
-      </c>
-      <c r="G16" s="10" t="inlineStr">
-        <is>
-          <t>one weld per 6 m stick — enter the number of sticks</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>76mm 304 press</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>3"</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>Straight</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="n"/>
-      <c r="E17" s="27">
-        <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B17,'Welding hours'!$C$3:$C$14,0),MATCH($C17,'Welding hours'!$D$2:$O$2,0)),0)</f>
-        <v/>
-      </c>
-      <c r="F17" s="27">
-        <f>D17*E17</f>
-        <v/>
-      </c>
-      <c r="G17" s="10" t="inlineStr">
-        <is>
-          <t>one weld per 6 m stick — enter the number of sticks</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>54mm 304 press</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>2"</t>
-        </is>
-      </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>Straight</t>
-        </is>
-      </c>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="27">
-        <f>IFERROR(INDEX('Welding hours'!$D$3:$O$14,MATCH($B18,'Welding hours'!$C$3:$C$14,0),MATCH($C18,'Welding hours'!$D$2:$O$2,0)),0)</f>
-        <v/>
-      </c>
-      <c r="F18" s="27">
-        <f>D18*E18</f>
-        <v/>
-      </c>
-      <c r="G18" s="10" t="inlineStr">
-        <is>
-          <t>one weld per 6 m stick — enter the number of sticks</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL WELDING HOURS</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="n"/>
-      <c r="C20" s="3" t="n"/>
-      <c r="D20" s="3" t="n"/>
-      <c r="E20" s="3" t="n"/>
-      <c r="F20" s="28">
-        <f>SUM(F2:F18)</f>
-        <v/>
-      </c>
-      <c r="G20" s="3" t="n"/>
+        <f>SUM(F2:F14)</f>
+        <v/>
+      </c>
+      <c r="G16" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5671,67 +5652,67 @@
   </cols>
   <sheetData>
     <row r="2">
-      <c r="C2" s="29" t="inlineStr">
+      <c r="C2" s="28" t="inlineStr">
         <is>
           <t>Rates</t>
         </is>
       </c>
-      <c r="D2" s="29" t="inlineStr">
+      <c r="D2" s="28" t="inlineStr">
         <is>
           <t>Weld Neck</t>
         </is>
       </c>
-      <c r="E2" s="29" t="inlineStr">
+      <c r="E2" s="28" t="inlineStr">
         <is>
           <t>Slip On</t>
         </is>
       </c>
-      <c r="F2" s="29" t="inlineStr">
+      <c r="F2" s="28" t="inlineStr">
         <is>
           <t>Blind</t>
         </is>
       </c>
-      <c r="G2" s="29" t="inlineStr">
+      <c r="G2" s="28" t="inlineStr">
         <is>
           <t>Socket Weld</t>
         </is>
       </c>
-      <c r="H2" s="29" t="inlineStr">
+      <c r="H2" s="28" t="inlineStr">
         <is>
           <t>Straight</t>
         </is>
       </c>
-      <c r="I2" s="29" t="inlineStr">
+      <c r="I2" s="28" t="inlineStr">
         <is>
           <t>Buttweld</t>
         </is>
       </c>
-      <c r="J2" s="29" t="inlineStr">
+      <c r="J2" s="28" t="inlineStr">
         <is>
           <t>Elbow</t>
         </is>
       </c>
-      <c r="K2" s="29" t="inlineStr">
+      <c r="K2" s="28" t="inlineStr">
         <is>
           <t>Tee</t>
         </is>
       </c>
-      <c r="L2" s="29" t="inlineStr">
+      <c r="L2" s="28" t="inlineStr">
         <is>
           <t>Reducer</t>
         </is>
       </c>
-      <c r="M2" s="29" t="inlineStr">
+      <c r="M2" s="28" t="inlineStr">
         <is>
           <t>Cap</t>
         </is>
       </c>
-      <c r="N2" s="29" t="inlineStr">
+      <c r="N2" s="28" t="inlineStr">
         <is>
           <t>Branch</t>
         </is>
       </c>
-      <c r="O2" s="29" t="inlineStr">
+      <c r="O2" s="28" t="inlineStr">
         <is>
           <t>Stab In</t>
         </is>

</xml_diff>

<commit_message>
quote-builder: drawings tidied, every run labelled with size + length (Riverbend-Q900142-Costing.xlsx)
</commit_message>
<xml_diff>
--- a/quote-builder/Riverbend-Q900142-Costing.xlsx
+++ b/quote-builder/Riverbend-Q900142-Costing.xlsx
@@ -566,7 +566,7 @@
         </is>
       </c>
       <c r="B8" s="4">
-        <f>Costing!K81</f>
+        <f>Costing!K79</f>
         <v/>
       </c>
     </row>
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15">
@@ -666,7 +666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L81"/>
+  <dimension ref="A1:L79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -964,7 +964,7 @@
     <row r="7">
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>65PN isolating valve</t>
+          <t>65TE isolating valve</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -974,7 +974,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>BF-65PN</t>
+          <t>BF-65TE</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr">
@@ -996,7 +996,7 @@
         </is>
       </c>
       <c r="I7" s="16" t="n">
-        <v>168</v>
+        <v>138</v>
       </c>
       <c r="J7" s="17" t="n">
         <v>0.15</v>
@@ -1007,14 +1007,14 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>1 × 65PN on the P&amp;ID</t>
+          <t>1 × 65TE on the P&amp;ID</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>65TE isolating valve</t>
+          <t>65PN isolating valve</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>BF-65TE</t>
+          <t>BF-65PN</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
@@ -1046,7 +1046,7 @@
         </is>
       </c>
       <c r="I8" s="16" t="n">
-        <v>138</v>
+        <v>168</v>
       </c>
       <c r="J8" s="17" t="n">
         <v>0.15</v>
@@ -1057,7 +1057,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>1 × 65TE on the P&amp;ID</t>
+          <t>1 × 65PN on the P&amp;ID</t>
         </is>
       </c>
     </row>
@@ -1779,190 +1779,190 @@
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="14" t="inlineStr">
+      <c r="B30" s="19" t="inlineStr">
+        <is>
+          <t>65TE tube flange</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>M-F</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="inlineStr"/>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>Bought in</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="inlineStr">
+        <is>
+          <t>RULE</t>
+        </is>
+      </c>
+      <c r="G30" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" s="10" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I30" s="20" t="n"/>
+      <c r="J30" s="21" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K30" s="20">
+        <f>IFERROR($G30*$I30,"")</f>
+        <v/>
+      </c>
+      <c r="L30" s="22" t="inlineStr">
+        <is>
+          <t>rule: 1 per 65TE connection</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>65TE gasket</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>M-F</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>GK-65</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>Bought in</t>
+        </is>
+      </c>
+      <c r="F31" s="15" t="inlineStr">
+        <is>
+          <t>PRICE LIST</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I31" s="16" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="J31" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K31" s="4">
+        <f>IFERROR($G31*$I31,"")</f>
+        <v/>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>rule: 1 per 65TE connection</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="14" t="inlineStr">
         <is>
           <t>65PN gasket</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>M-F</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>GK-65</t>
         </is>
       </c>
-      <c r="E30" s="10" t="inlineStr">
+      <c r="E32" s="10" t="inlineStr">
         <is>
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F30" s="15" t="inlineStr">
+      <c r="F32" s="15" t="inlineStr">
         <is>
           <t>PRICE LIST</t>
         </is>
       </c>
-      <c r="G30" t="n">
+      <c r="G32" t="n">
         <v>1</v>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="I30" s="16" t="n">
+      <c r="I32" s="16" t="n">
         <v>5.4</v>
       </c>
-      <c r="J30" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K30" s="4">
-        <f>IFERROR($G30*$I30,"")</f>
-        <v/>
-      </c>
-      <c r="L30" s="2" t="inlineStr">
+      <c r="J32" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K32" s="4">
+        <f>IFERROR($G32*$I32,"")</f>
+        <v/>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
         <is>
           <t>rule: 1 per 65PN connection</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="19" t="inlineStr">
+    <row r="33">
+      <c r="B33" s="19" t="inlineStr">
         <is>
           <t>65PN bolt set</t>
         </is>
       </c>
-      <c r="C31" s="10" t="inlineStr">
+      <c r="C33" s="10" t="inlineStr">
         <is>
           <t>M-F</t>
         </is>
       </c>
-      <c r="D31" s="10" t="inlineStr"/>
-      <c r="E31" s="10" t="inlineStr">
+      <c r="D33" s="10" t="inlineStr"/>
+      <c r="E33" s="10" t="inlineStr">
         <is>
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F31" s="10" t="inlineStr">
+      <c r="F33" s="10" t="inlineStr">
         <is>
           <t>RULE</t>
         </is>
       </c>
-      <c r="G31" s="10" t="n">
+      <c r="G33" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="H31" s="10" t="inlineStr">
+      <c r="H33" s="10" t="inlineStr">
         <is>
           <t>ea</t>
         </is>
       </c>
-      <c r="I31" s="20" t="n"/>
-      <c r="J31" s="21" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K31" s="20">
-        <f>IFERROR($G31*$I31,"")</f>
-        <v/>
-      </c>
-      <c r="L31" s="22" t="inlineStr">
+      <c r="I33" s="20" t="n"/>
+      <c r="J33" s="21" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K33" s="20">
+        <f>IFERROR($G33*$I33,"")</f>
+        <v/>
+      </c>
+      <c r="L33" s="22" t="inlineStr">
         <is>
           <t>rule: 1 per 65PN connection</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="19" t="inlineStr">
-        <is>
-          <t>65TE tube flange</t>
-        </is>
-      </c>
-      <c r="C32" s="10" t="inlineStr">
-        <is>
-          <t>M-F</t>
-        </is>
-      </c>
-      <c r="D32" s="10" t="inlineStr"/>
-      <c r="E32" s="10" t="inlineStr">
-        <is>
-          <t>Bought in</t>
-        </is>
-      </c>
-      <c r="F32" s="10" t="inlineStr">
-        <is>
-          <t>RULE</t>
-        </is>
-      </c>
-      <c r="G32" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H32" s="10" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I32" s="20" t="n"/>
-      <c r="J32" s="21" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K32" s="20">
-        <f>IFERROR($G32*$I32,"")</f>
-        <v/>
-      </c>
-      <c r="L32" s="22" t="inlineStr">
-        <is>
-          <t>rule: 1 per 65TE connection</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="14" t="inlineStr">
-        <is>
-          <t>65TE gasket</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>M-F</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>GK-65</t>
-        </is>
-      </c>
-      <c r="E33" s="10" t="inlineStr">
-        <is>
-          <t>Bought in</t>
-        </is>
-      </c>
-      <c r="F33" s="15" t="inlineStr">
-        <is>
-          <t>PRICE LIST</t>
-        </is>
-      </c>
-      <c r="G33" t="n">
-        <v>1</v>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I33" s="16" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="J33" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K33" s="4">
-        <f>IFERROR($G33*$I33,"")</f>
-        <v/>
-      </c>
-      <c r="L33" s="2" t="inlineStr">
-        <is>
-          <t>rule: 1 per 65TE connection</t>
         </is>
       </c>
     </row>
@@ -2107,34 +2107,40 @@
     <row r="37">
       <c r="B37" s="14" t="inlineStr">
         <is>
-          <t>50NB pipe</t>
+          <t>76mm 304 press pipe</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>M-P</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr"/>
+          <t>M-PFS</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>PT-76</t>
+        </is>
+      </c>
       <c r="E37" s="10" t="inlineStr">
         <is>
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>ENGINEER</t>
+      <c r="F37" s="15" t="inlineStr">
+        <is>
+          <t>PRICE LIST</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="I37" s="4" t="n"/>
+      <c r="I37" s="16" t="n">
+        <v>53.1</v>
+      </c>
       <c r="J37" s="17" t="n">
         <v>0.15</v>
       </c>
@@ -2144,41 +2150,47 @@
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>1 run on the P&amp;ID · 45 m off the drawing = 45 m</t>
+          <t>1 run on the P&amp;ID · 10 m off the drawing = 10 m</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>101mm tube pipe</t>
+          <t>54mm 304 press pipe</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>M-P</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr"/>
+          <t>M-PFS</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>PT-54</t>
+        </is>
+      </c>
       <c r="E38" s="10" t="inlineStr">
         <is>
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>ENGINEER</t>
+      <c r="F38" s="15" t="inlineStr">
+        <is>
+          <t>PRICE LIST</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="I38" s="4" t="n"/>
+      <c r="I38" s="16" t="n">
+        <v>17.4</v>
+      </c>
       <c r="J38" s="17" t="n">
         <v>0.15</v>
       </c>
@@ -2188,14 +2200,14 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>1 run on the P&amp;ID · 12 m off the drawing = 12 m</t>
+          <t>1 run on the P&amp;ID · 10 m off the drawing = 10 m</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>63mm tube pipe</t>
+          <t>50NB pipe</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2215,7 +2227,7 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -2232,97 +2244,82 @@
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>1 run on the P&amp;ID · 12 m off the drawing = 12 m</t>
+          <t>1 run on the P&amp;ID · 45 m off the drawing = 45 m</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="14" t="inlineStr">
-        <is>
-          <t>76mm 304 press pipe</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>M-PFS</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>PT-76</t>
-        </is>
-      </c>
+      <c r="B40" s="19" t="inlineStr">
+        <is>
+          <t>Pipe insulation</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t>M-INS</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="inlineStr"/>
       <c r="E40" s="10" t="inlineStr">
         <is>
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F40" s="15" t="inlineStr">
-        <is>
-          <t>PRICE LIST</t>
-        </is>
-      </c>
-      <c r="G40" t="n">
-        <v>10</v>
-      </c>
-      <c r="H40" t="inlineStr">
+      <c r="F40" s="10" t="inlineStr">
+        <is>
+          <t>RATE</t>
+        </is>
+      </c>
+      <c r="G40" s="10" t="n">
+        <v>219</v>
+      </c>
+      <c r="H40" s="10" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="I40" s="16" t="n">
-        <v>53.1</v>
-      </c>
-      <c r="J40" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K40" s="4">
+      <c r="I40" s="20" t="n"/>
+      <c r="J40" s="21" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K40" s="20">
         <f>IFERROR($G40*$I40,"")</f>
         <v/>
       </c>
-      <c r="L40" s="2" t="inlineStr">
-        <is>
-          <t>1 run on the P&amp;ID · 10 m off the drawing = 10 m</t>
+      <c r="L40" s="22" t="inlineStr">
+        <is>
+          <t>15 insulated runs · 219 m off the drawing (drains excluded)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="14" t="inlineStr">
         <is>
-          <t>54mm 304 press pipe</t>
+          <t>Freight and cartage</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>M-PFS</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>PT-54</t>
-        </is>
-      </c>
+          <t>P-FRE</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
       <c r="E41" s="10" t="inlineStr">
         <is>
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F41" s="15" t="inlineStr">
-        <is>
-          <t>PRICE LIST</t>
-        </is>
-      </c>
-      <c r="G41" t="n">
-        <v>10</v>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>ENGINEER</t>
+        </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="I41" s="16" t="n">
-        <v>17.4</v>
-      </c>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="I41" s="4" t="n"/>
       <c r="J41" s="17" t="n">
         <v>0.15</v>
       </c>
@@ -2332,142 +2329,143 @@
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>1 run on the P&amp;ID · 10 m off the drawing = 10 m</t>
+          <t>carried on past jobs</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="19" t="inlineStr">
-        <is>
-          <t>Pipe insulation</t>
-        </is>
-      </c>
-      <c r="C42" s="10" t="inlineStr">
-        <is>
-          <t>M-INS</t>
-        </is>
-      </c>
-      <c r="D42" s="10" t="inlineStr"/>
-      <c r="E42" s="10" t="inlineStr">
-        <is>
-          <t>Bought in</t>
-        </is>
-      </c>
-      <c r="F42" s="10" t="inlineStr">
-        <is>
-          <t>RATE</t>
-        </is>
-      </c>
-      <c r="G42" s="10" t="n">
-        <v>243</v>
-      </c>
-      <c r="H42" s="10" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="I42" s="20" t="n"/>
-      <c r="J42" s="21" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K42" s="20">
-        <f>IFERROR($G42*$I42,"")</f>
-        <v/>
-      </c>
-      <c r="L42" s="22" t="inlineStr">
-        <is>
-          <t>17 insulated runs · 243 m off the drawing (drains excluded)</t>
-        </is>
-      </c>
+      <c r="A42" s="3" t="n"/>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Section 7.6 total</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="n"/>
+      <c r="D42" s="3" t="n"/>
+      <c r="E42" s="3" t="n"/>
+      <c r="F42" s="3" t="n"/>
+      <c r="G42" s="3" t="n"/>
+      <c r="H42" s="3" t="n"/>
+      <c r="I42" s="3" t="n"/>
+      <c r="J42" s="3" t="n"/>
+      <c r="K42" s="18">
+        <f>SUM(K24:K41)</f>
+        <v/>
+      </c>
+      <c r="L42" s="3" t="n"/>
     </row>
     <row r="43">
-      <c r="B43" s="14" t="inlineStr">
-        <is>
-          <t>Freight and cartage</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>P-FRE</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" s="10" t="inlineStr">
-        <is>
-          <t>Bought in</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>7.7</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Installation labour, supervision and consumables</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="n"/>
+      <c r="D43" s="7" t="n"/>
+      <c r="E43" s="7" t="n"/>
+      <c r="F43" s="7" t="n"/>
+      <c r="G43" s="7" t="n"/>
+      <c r="H43" s="7" t="n"/>
+      <c r="I43" s="7" t="n"/>
+      <c r="J43" s="7" t="n"/>
+      <c r="K43" s="7" t="n"/>
+      <c r="L43" s="7" t="n"/>
+    </row>
+    <row r="44">
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>Set out and rig plant</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>L-SERVIN</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" s="15" t="inlineStr">
+        <is>
+          <t>In-house</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
         <is>
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>lot</t>
-        </is>
-      </c>
-      <c r="I43" s="4" t="n"/>
-      <c r="J43" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K43" s="4">
-        <f>IFERROR($G43*$I43,"")</f>
-        <v/>
-      </c>
-      <c r="L43" s="2" t="inlineStr">
-        <is>
-          <t>carried on past jobs</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="3" t="n"/>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>Section 7.6 total</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="n"/>
-      <c r="D44" s="3" t="n"/>
-      <c r="E44" s="3" t="n"/>
-      <c r="F44" s="3" t="n"/>
-      <c r="G44" s="3" t="n"/>
-      <c r="H44" s="3" t="n"/>
-      <c r="I44" s="3" t="n"/>
-      <c r="J44" s="3" t="n"/>
-      <c r="K44" s="18">
-        <f>SUM(K24:K43)</f>
-        <v/>
-      </c>
-      <c r="L44" s="3" t="n"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="I44" s="4" t="n">
+        <v>105</v>
+      </c>
+      <c r="J44" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K44" s="4">
+        <f>IFERROR($G44*$I44,"")</f>
+        <v/>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>crew × days</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
-        <is>
-          <t>7.7</t>
-        </is>
-      </c>
-      <c r="B45" s="7" t="inlineStr">
-        <is>
-          <t>Installation labour, supervision and consumables</t>
-        </is>
-      </c>
-      <c r="C45" s="7" t="n"/>
-      <c r="D45" s="7" t="n"/>
-      <c r="E45" s="7" t="n"/>
-      <c r="F45" s="7" t="n"/>
-      <c r="G45" s="7" t="n"/>
-      <c r="H45" s="7" t="n"/>
-      <c r="I45" s="7" t="n"/>
-      <c r="J45" s="7" t="n"/>
-      <c r="K45" s="7" t="n"/>
-      <c r="L45" s="7" t="n"/>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>Pipe compressor pack</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>L-SERVIN</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" s="15" t="inlineStr">
+        <is>
+          <t>In-house</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>ENGINEER</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="n">
+        <v>105</v>
+      </c>
+      <c r="J45" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K45" s="4">
+        <f>IFERROR($G45*$I45,"")</f>
+        <v/>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>crew × days</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="B46" s="14" t="inlineStr">
         <is>
-          <t>Set out and rig plant</t>
+          <t>Pipe chiller and glycol circuit</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2510,7 +2508,7 @@
     <row r="47">
       <c r="B47" s="14" t="inlineStr">
         <is>
-          <t>Pipe compressor pack</t>
+          <t>Hang and pipe unit coolers</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2553,7 +2551,7 @@
     <row r="48">
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>Pipe chiller and glycol circuit</t>
+          <t>Pressure test</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2596,7 +2594,7 @@
     <row r="49">
       <c r="B49" s="14" t="inlineStr">
         <is>
-          <t>Hang and pipe unit coolers</t>
+          <t>Insulate</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2639,7 +2637,7 @@
     <row r="50">
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t>Pressure test</t>
+          <t>Glycol fill and flush</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2682,7 +2680,7 @@
     <row r="51">
       <c r="B51" s="14" t="inlineStr">
         <is>
-          <t>Insulate</t>
+          <t>Changeover weekend</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2725,7 +2723,7 @@
     <row r="52">
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>Glycol fill and flush</t>
+          <t>Supervision</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2768,18 +2766,18 @@
     <row r="53">
       <c r="B53" s="14" t="inlineStr">
         <is>
-          <t>Changeover weekend</t>
+          <t>Crane and access hire</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>L-SERVIN</t>
+          <t>P-HIRE</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
-      <c r="E53" s="15" t="inlineStr">
-        <is>
-          <t>In-house</t>
+      <c r="E53" s="10" t="inlineStr">
+        <is>
+          <t>Bought in</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2789,12 +2787,10 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>hr</t>
-        </is>
-      </c>
-      <c r="I53" s="4" t="n">
-        <v>105</v>
-      </c>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="I53" s="4" t="n"/>
       <c r="J53" s="17" t="n">
         <v>0.15</v>
       </c>
@@ -2804,25 +2800,25 @@
       </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>crew × days</t>
+          <t>carried on past jobs</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>Supervision</t>
+          <t>Travel and accommodation</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>L-SERVIN</t>
+          <t>D-TRAV</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
-      <c r="E54" s="15" t="inlineStr">
-        <is>
-          <t>In-house</t>
+      <c r="E54" s="10" t="inlineStr">
+        <is>
+          <t>Bought in</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2832,12 +2828,10 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>hr</t>
-        </is>
-      </c>
-      <c r="I54" s="4" t="n">
-        <v>105</v>
-      </c>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="I54" s="4" t="n"/>
       <c r="J54" s="17" t="n">
         <v>0.15</v>
       </c>
@@ -2847,19 +2841,19 @@
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>crew × days</t>
+          <t>carried on past jobs</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="B55" s="14" t="inlineStr">
         <is>
-          <t>Crane and access hire</t>
+          <t>Site setup and safety</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>P-HIRE</t>
+          <t>P-SS</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -2893,312 +2887,316 @@
       </c>
     </row>
     <row r="56">
-      <c r="B56" s="14" t="inlineStr">
-        <is>
-          <t>Travel and accommodation</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>D-TRAV</t>
+      <c r="B56" s="15" t="inlineStr">
+        <is>
+          <t>Site welding and fit-up</t>
+        </is>
+      </c>
+      <c r="C56" s="15" t="inlineStr">
+        <is>
+          <t>L-SERVIN</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
-      <c r="E56" s="10" t="inlineStr">
-        <is>
-          <t>Bought in</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
+      <c r="E56" s="15" t="inlineStr">
+        <is>
+          <t>In-house</t>
+        </is>
+      </c>
+      <c r="F56" s="15" t="inlineStr">
+        <is>
+          <t>TAKE-OFF</t>
+        </is>
+      </c>
+      <c r="G56" s="23">
+        <f>'Take-off'!F16</f>
+        <v/>
+      </c>
+      <c r="H56" s="15" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="I56" s="16" t="n">
+        <v>110</v>
+      </c>
+      <c r="J56" s="24" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K56" s="16">
+        <f>IFERROR($G56*$I56,"")</f>
+        <v/>
+      </c>
+      <c r="L56" s="25" t="inlineStr">
+        <is>
+          <t>hours from the Take-off, priced off the Welding hours matrix</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="n"/>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Section 7.7 total</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="n"/>
+      <c r="D57" s="3" t="n"/>
+      <c r="E57" s="3" t="n"/>
+      <c r="F57" s="3" t="n"/>
+      <c r="G57" s="3" t="n"/>
+      <c r="H57" s="3" t="n"/>
+      <c r="I57" s="3" t="n"/>
+      <c r="J57" s="3" t="n"/>
+      <c r="K57" s="18">
+        <f>SUM(K44:K56)</f>
+        <v/>
+      </c>
+      <c r="L57" s="3" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>7.8</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Electrical power, control wiring and SCADA</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="n"/>
+      <c r="D58" s="7" t="n"/>
+      <c r="E58" s="7" t="n"/>
+      <c r="F58" s="7" t="n"/>
+      <c r="G58" s="7" t="n"/>
+      <c r="H58" s="7" t="n"/>
+      <c r="I58" s="7" t="n"/>
+      <c r="J58" s="7" t="n"/>
+      <c r="K58" s="7" t="n"/>
+      <c r="L58" s="7" t="n"/>
+    </row>
+    <row r="59">
+      <c r="B59" s="8" t="inlineStr">
+        <is>
+          <t>Power and control wiring</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr">
+        <is>
+          <t>ES-INST</t>
+        </is>
+      </c>
+      <c r="D59" s="9" t="inlineStr"/>
+      <c r="E59" s="9" t="inlineStr">
+        <is>
+          <t>Subcontract</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="inlineStr">
+        <is>
+          <t>RFQ</t>
+        </is>
+      </c>
+      <c r="G59" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H59" s="9" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="I59" s="11" t="n"/>
+      <c r="J59" s="12" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K59" s="11">
+        <f>IFERROR($G59*$I59,"")</f>
+        <v/>
+      </c>
+      <c r="L59" s="13" t="inlineStr">
+        <is>
+          <t>from the maximum demand schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>SCADA integration — Ignition</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="inlineStr">
+        <is>
+          <t>ES-AU</t>
+        </is>
+      </c>
+      <c r="D60" s="9" t="inlineStr"/>
+      <c r="E60" s="9" t="inlineStr">
+        <is>
+          <t>Subcontract</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="inlineStr">
+        <is>
+          <t>RFQ</t>
+        </is>
+      </c>
+      <c r="G60" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H60" s="9" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="I60" s="11" t="n"/>
+      <c r="J60" s="12" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K60" s="11">
+        <f>IFERROR($G60*$I60,"")</f>
+        <v/>
+      </c>
+      <c r="L60" s="13" t="inlineStr">
+        <is>
+          <t>electrical contractor</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="n"/>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Section 7.8 total</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="n"/>
+      <c r="D61" s="3" t="n"/>
+      <c r="E61" s="3" t="n"/>
+      <c r="F61" s="3" t="n"/>
+      <c r="G61" s="3" t="n"/>
+      <c r="H61" s="3" t="n"/>
+      <c r="I61" s="3" t="n"/>
+      <c r="J61" s="3" t="n"/>
+      <c r="K61" s="18">
+        <f>SUM(K59:K60)</f>
+        <v/>
+      </c>
+      <c r="L61" s="3" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>7.9</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>As-built documentation, training, O&amp;M</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="n"/>
+      <c r="D62" s="7" t="n"/>
+      <c r="E62" s="7" t="n"/>
+      <c r="F62" s="7" t="n"/>
+      <c r="G62" s="7" t="n"/>
+      <c r="H62" s="7" t="n"/>
+      <c r="I62" s="7" t="n"/>
+      <c r="J62" s="7" t="n"/>
+      <c r="K62" s="7" t="n"/>
+      <c r="L62" s="7" t="n"/>
+    </row>
+    <row r="63">
+      <c r="B63" s="14" t="inlineStr">
+        <is>
+          <t>As-built drawings</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>L-DWG</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" s="15" t="inlineStr">
+        <is>
+          <t>In-house</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
         <is>
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>lot</t>
-        </is>
-      </c>
-      <c r="I56" s="4" t="n"/>
-      <c r="J56" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K56" s="4">
-        <f>IFERROR($G56*$I56,"")</f>
-        <v/>
-      </c>
-      <c r="L56" s="2" t="inlineStr">
-        <is>
-          <t>carried on past jobs</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="B57" s="14" t="inlineStr">
-        <is>
-          <t>Site setup and safety</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>P-SS</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" s="10" t="inlineStr">
-        <is>
-          <t>Bought in</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="I63" s="4" t="n">
+        <v>140</v>
+      </c>
+      <c r="J63" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K63" s="4">
+        <f>IFERROR($G63*$I63,"")</f>
+        <v/>
+      </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>hours to be entered</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="14" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>L-DWG</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" s="15" t="inlineStr">
+        <is>
+          <t>In-house</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
         <is>
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>lot</t>
-        </is>
-      </c>
-      <c r="I57" s="4" t="n"/>
-      <c r="J57" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K57" s="4">
-        <f>IFERROR($G57*$I57,"")</f>
-        <v/>
-      </c>
-      <c r="L57" s="2" t="inlineStr">
-        <is>
-          <t>carried on past jobs</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="B58" s="15" t="inlineStr">
-        <is>
-          <t>Site welding and fit-up</t>
-        </is>
-      </c>
-      <c r="C58" s="15" t="inlineStr">
-        <is>
-          <t>L-SERVIN</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" s="15" t="inlineStr">
-        <is>
-          <t>In-house</t>
-        </is>
-      </c>
-      <c r="F58" s="15" t="inlineStr">
-        <is>
-          <t>TAKE-OFF</t>
-        </is>
-      </c>
-      <c r="G58" s="23">
-        <f>'Take-off'!F16</f>
-        <v/>
-      </c>
-      <c r="H58" s="15" t="inlineStr">
+      <c r="H64" t="inlineStr">
         <is>
           <t>hr</t>
         </is>
       </c>
-      <c r="I58" s="16" t="n">
-        <v>110</v>
-      </c>
-      <c r="J58" s="24" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K58" s="16">
-        <f>IFERROR($G58*$I58,"")</f>
-        <v/>
-      </c>
-      <c r="L58" s="25" t="inlineStr">
-        <is>
-          <t>hours from the Take-off, priced off the Welding hours matrix</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="3" t="n"/>
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>Section 7.7 total</t>
-        </is>
-      </c>
-      <c r="C59" s="3" t="n"/>
-      <c r="D59" s="3" t="n"/>
-      <c r="E59" s="3" t="n"/>
-      <c r="F59" s="3" t="n"/>
-      <c r="G59" s="3" t="n"/>
-      <c r="H59" s="3" t="n"/>
-      <c r="I59" s="3" t="n"/>
-      <c r="J59" s="3" t="n"/>
-      <c r="K59" s="18">
-        <f>SUM(K46:K58)</f>
-        <v/>
-      </c>
-      <c r="L59" s="3" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="7" t="inlineStr">
-        <is>
-          <t>7.8</t>
-        </is>
-      </c>
-      <c r="B60" s="7" t="inlineStr">
-        <is>
-          <t>Electrical power, control wiring and SCADA</t>
-        </is>
-      </c>
-      <c r="C60" s="7" t="n"/>
-      <c r="D60" s="7" t="n"/>
-      <c r="E60" s="7" t="n"/>
-      <c r="F60" s="7" t="n"/>
-      <c r="G60" s="7" t="n"/>
-      <c r="H60" s="7" t="n"/>
-      <c r="I60" s="7" t="n"/>
-      <c r="J60" s="7" t="n"/>
-      <c r="K60" s="7" t="n"/>
-      <c r="L60" s="7" t="n"/>
-    </row>
-    <row r="61">
-      <c r="B61" s="8" t="inlineStr">
-        <is>
-          <t>Power and control wiring</t>
-        </is>
-      </c>
-      <c r="C61" s="9" t="inlineStr">
-        <is>
-          <t>ES-INST</t>
-        </is>
-      </c>
-      <c r="D61" s="9" t="inlineStr"/>
-      <c r="E61" s="9" t="inlineStr">
-        <is>
-          <t>Subcontract</t>
-        </is>
-      </c>
-      <c r="F61" s="9" t="inlineStr">
-        <is>
-          <t>RFQ</t>
-        </is>
-      </c>
-      <c r="G61" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="H61" s="9" t="inlineStr">
-        <is>
-          <t>lot</t>
-        </is>
-      </c>
-      <c r="I61" s="11" t="n"/>
-      <c r="J61" s="12" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K61" s="11">
-        <f>IFERROR($G61*$I61,"")</f>
-        <v/>
-      </c>
-      <c r="L61" s="13" t="inlineStr">
-        <is>
-          <t>from the maximum demand schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="B62" s="8" t="inlineStr">
-        <is>
-          <t>SCADA integration — Ignition</t>
-        </is>
-      </c>
-      <c r="C62" s="9" t="inlineStr">
-        <is>
-          <t>ES-AU</t>
-        </is>
-      </c>
-      <c r="D62" s="9" t="inlineStr"/>
-      <c r="E62" s="9" t="inlineStr">
-        <is>
-          <t>Subcontract</t>
-        </is>
-      </c>
-      <c r="F62" s="9" t="inlineStr">
-        <is>
-          <t>RFQ</t>
-        </is>
-      </c>
-      <c r="G62" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="H62" s="9" t="inlineStr">
-        <is>
-          <t>lot</t>
-        </is>
-      </c>
-      <c r="I62" s="11" t="n"/>
-      <c r="J62" s="12" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K62" s="11">
-        <f>IFERROR($G62*$I62,"")</f>
-        <v/>
-      </c>
-      <c r="L62" s="13" t="inlineStr">
-        <is>
-          <t>electrical contractor</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="3" t="n"/>
-      <c r="B63" s="3" t="inlineStr">
-        <is>
-          <t>Section 7.8 total</t>
-        </is>
-      </c>
-      <c r="C63" s="3" t="n"/>
-      <c r="D63" s="3" t="n"/>
-      <c r="E63" s="3" t="n"/>
-      <c r="F63" s="3" t="n"/>
-      <c r="G63" s="3" t="n"/>
-      <c r="H63" s="3" t="n"/>
-      <c r="I63" s="3" t="n"/>
-      <c r="J63" s="3" t="n"/>
-      <c r="K63" s="18">
-        <f>SUM(K61:K62)</f>
-        <v/>
-      </c>
-      <c r="L63" s="3" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="7" t="inlineStr">
-        <is>
-          <t>7.9</t>
-        </is>
-      </c>
-      <c r="B64" s="7" t="inlineStr">
-        <is>
-          <t>As-built documentation, training, O&amp;M</t>
-        </is>
-      </c>
-      <c r="C64" s="7" t="n"/>
-      <c r="D64" s="7" t="n"/>
-      <c r="E64" s="7" t="n"/>
-      <c r="F64" s="7" t="n"/>
-      <c r="G64" s="7" t="n"/>
-      <c r="H64" s="7" t="n"/>
-      <c r="I64" s="7" t="n"/>
-      <c r="J64" s="7" t="n"/>
-      <c r="K64" s="7" t="n"/>
-      <c r="L64" s="7" t="n"/>
+      <c r="I64" s="4" t="n">
+        <v>140</v>
+      </c>
+      <c r="J64" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K64" s="4">
+        <f>IFERROR($G64*$I64,"")</f>
+        <v/>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>hours to be entered</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="B65" s="14" t="inlineStr">
         <is>
-          <t>As-built drawings</t>
+          <t>O&amp;M manuals</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3241,12 +3239,12 @@
     <row r="66">
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Producer statements</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>L-DWG</t>
+          <t>L-DV</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -3284,18 +3282,18 @@
     <row r="67">
       <c r="B67" s="14" t="inlineStr">
         <is>
-          <t>O&amp;M manuals</t>
+          <t>Compliance and inspection</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>L-DWG</t>
+          <t>P-RCOMP</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
-      <c r="E67" s="15" t="inlineStr">
-        <is>
-          <t>In-house</t>
+      <c r="E67" s="10" t="inlineStr">
+        <is>
+          <t>Bought in</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -3305,12 +3303,10 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>hr</t>
-        </is>
-      </c>
-      <c r="I67" s="4" t="n">
-        <v>140</v>
-      </c>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="I67" s="4" t="n"/>
       <c r="J67" s="17" t="n">
         <v>0.15</v>
       </c>
@@ -3320,152 +3316,152 @@
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>hours to be entered</t>
+          <t>carried on past jobs</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="B68" s="14" t="inlineStr">
-        <is>
-          <t>Producer statements</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>L-DV</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" s="15" t="inlineStr">
+      <c r="A68" s="3" t="n"/>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Section 7.9 total</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="n"/>
+      <c r="D68" s="3" t="n"/>
+      <c r="E68" s="3" t="n"/>
+      <c r="F68" s="3" t="n"/>
+      <c r="G68" s="3" t="n"/>
+      <c r="H68" s="3" t="n"/>
+      <c r="I68" s="3" t="n"/>
+      <c r="J68" s="3" t="n"/>
+      <c r="K68" s="18">
+        <f>SUM(K63:K67)</f>
+        <v/>
+      </c>
+      <c r="L68" s="3" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="7" t="inlineStr">
+        <is>
+          <t>7.10</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>Commissioning, glycol charge and spares</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="n"/>
+      <c r="D69" s="7" t="n"/>
+      <c r="E69" s="7" t="n"/>
+      <c r="F69" s="7" t="n"/>
+      <c r="G69" s="7" t="n"/>
+      <c r="H69" s="7" t="n"/>
+      <c r="I69" s="7" t="n"/>
+      <c r="J69" s="7" t="n"/>
+      <c r="K69" s="7" t="n"/>
+      <c r="L69" s="7" t="n"/>
+    </row>
+    <row r="70">
+      <c r="B70" s="14" t="inlineStr">
+        <is>
+          <t>Commissioning and pulldown demonstration</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>L-COM</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" s="15" t="inlineStr">
         <is>
           <t>In-house</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr">
+      <c r="F70" t="inlineStr">
         <is>
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr">
+      <c r="H70" t="inlineStr">
         <is>
           <t>hr</t>
         </is>
       </c>
-      <c r="I68" s="4" t="n">
-        <v>140</v>
-      </c>
-      <c r="J68" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K68" s="4">
-        <f>IFERROR($G68*$I68,"")</f>
-        <v/>
-      </c>
-      <c r="L68" s="2" t="inlineStr">
-        <is>
-          <t>hours to be entered</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="B69" s="14" t="inlineStr">
-        <is>
-          <t>Compliance and inspection</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>P-RCOMP</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" s="10" t="inlineStr">
+      <c r="I70" s="4" t="n">
+        <v>105</v>
+      </c>
+      <c r="J70" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K70" s="4">
+        <f>IFERROR($G70*$I70,"")</f>
+        <v/>
+      </c>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>to be entered</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="14" t="inlineStr">
+        <is>
+          <t>Glycol charge — MPG 35%</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>R-GLY</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" s="10" t="inlineStr">
         <is>
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="F71" t="inlineStr">
         <is>
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>lot</t>
-        </is>
-      </c>
-      <c r="I69" s="4" t="n"/>
-      <c r="J69" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K69" s="4">
-        <f>IFERROR($G69*$I69,"")</f>
-        <v/>
-      </c>
-      <c r="L69" s="2" t="inlineStr">
-        <is>
-          <t>carried on past jobs</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="3" t="n"/>
-      <c r="B70" s="3" t="inlineStr">
-        <is>
-          <t>Section 7.9 total</t>
-        </is>
-      </c>
-      <c r="C70" s="3" t="n"/>
-      <c r="D70" s="3" t="n"/>
-      <c r="E70" s="3" t="n"/>
-      <c r="F70" s="3" t="n"/>
-      <c r="G70" s="3" t="n"/>
-      <c r="H70" s="3" t="n"/>
-      <c r="I70" s="3" t="n"/>
-      <c r="J70" s="3" t="n"/>
-      <c r="K70" s="18">
-        <f>SUM(K65:K69)</f>
-        <v/>
-      </c>
-      <c r="L70" s="3" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="7" t="inlineStr">
-        <is>
-          <t>7.10</t>
-        </is>
-      </c>
-      <c r="B71" s="7" t="inlineStr">
-        <is>
-          <t>Commissioning, glycol charge and spares</t>
-        </is>
-      </c>
-      <c r="C71" s="7" t="n"/>
-      <c r="D71" s="7" t="n"/>
-      <c r="E71" s="7" t="n"/>
-      <c r="F71" s="7" t="n"/>
-      <c r="G71" s="7" t="n"/>
-      <c r="H71" s="7" t="n"/>
-      <c r="I71" s="7" t="n"/>
-      <c r="J71" s="7" t="n"/>
-      <c r="K71" s="7" t="n"/>
-      <c r="L71" s="7" t="n"/>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I71" s="4" t="n"/>
+      <c r="J71" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K71" s="4">
+        <f>IFERROR($G71*$I71,"")</f>
+        <v/>
+      </c>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>to be entered</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="B72" s="14" t="inlineStr">
         <is>
-          <t>Commissioning and pulldown demonstration</t>
+          <t>Spare parts</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>L-COM</t>
+          <t>M-GEN</t>
         </is>
       </c>
       <c r="D72" t="inlineStr"/>
-      <c r="E72" s="15" t="inlineStr">
-        <is>
-          <t>In-house</t>
+      <c r="E72" s="10" t="inlineStr">
+        <is>
+          <t>Bought in</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3475,12 +3471,10 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>hr</t>
-        </is>
-      </c>
-      <c r="I72" s="4" t="n">
-        <v>105</v>
-      </c>
+          <t>ea</t>
+        </is>
+      </c>
+      <c r="I72" s="4" t="n"/>
       <c r="J72" s="17" t="n">
         <v>0.15</v>
       </c>
@@ -3495,220 +3489,159 @@
       </c>
     </row>
     <row r="73">
-      <c r="B73" s="14" t="inlineStr">
-        <is>
-          <t>Glycol charge — MPG 35%</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>R-GLY</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr"/>
-      <c r="E73" s="10" t="inlineStr">
+      <c r="A73" s="3" t="n"/>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>Section 7.10 total</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="n"/>
+      <c r="D73" s="3" t="n"/>
+      <c r="E73" s="3" t="n"/>
+      <c r="F73" s="3" t="n"/>
+      <c r="G73" s="3" t="n"/>
+      <c r="H73" s="3" t="n"/>
+      <c r="I73" s="3" t="n"/>
+      <c r="J73" s="3" t="n"/>
+      <c r="K73" s="18">
+        <f>SUM(K70:K72)</f>
+        <v/>
+      </c>
+      <c r="L73" s="3" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="7" t="inlineStr">
+        <is>
+          <t>7.11</t>
+        </is>
+      </c>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>Twelve months defects liability and routine maintenance</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="n"/>
+      <c r="D74" s="7" t="n"/>
+      <c r="E74" s="7" t="n"/>
+      <c r="F74" s="7" t="n"/>
+      <c r="G74" s="7" t="n"/>
+      <c r="H74" s="7" t="n"/>
+      <c r="I74" s="7" t="n"/>
+      <c r="J74" s="7" t="n"/>
+      <c r="K74" s="7" t="n"/>
+      <c r="L74" s="7" t="n"/>
+    </row>
+    <row r="75">
+      <c r="B75" s="14" t="inlineStr">
+        <is>
+          <t>Routine maintenance, 12 months</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>D-MAINT</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" s="10" t="inlineStr">
         <is>
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr">
+      <c r="F75" t="inlineStr">
         <is>
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="I73" s="4" t="n"/>
-      <c r="J73" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K73" s="4">
-        <f>IFERROR($G73*$I73,"")</f>
-        <v/>
-      </c>
-      <c r="L73" s="2" t="inlineStr">
-        <is>
-          <t>to be entered</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="B74" s="14" t="inlineStr">
-        <is>
-          <t>Spare parts</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>M-GEN</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr"/>
-      <c r="E74" s="10" t="inlineStr">
+      <c r="G75" t="n">
+        <v>4</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>visit</t>
+        </is>
+      </c>
+      <c r="I75" s="4" t="n"/>
+      <c r="J75" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K75" s="4">
+        <f>IFERROR($G75*$I75,"")</f>
+        <v/>
+      </c>
+      <c r="L75" s="2" t="inlineStr">
+        <is>
+          <t>rate to be entered</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="14" t="inlineStr">
+        <is>
+          <t>Contingency</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>D-CONT</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" s="10" t="inlineStr">
         <is>
           <t>Bought in</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr">
+      <c r="F76" t="inlineStr">
         <is>
           <t>ENGINEER</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>ea</t>
-        </is>
-      </c>
-      <c r="I74" s="4" t="n"/>
-      <c r="J74" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K74" s="4">
-        <f>IFERROR($G74*$I74,"")</f>
-        <v/>
-      </c>
-      <c r="L74" s="2" t="inlineStr">
-        <is>
-          <t>to be entered</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="3" t="n"/>
-      <c r="B75" s="3" t="inlineStr">
-        <is>
-          <t>Section 7.10 total</t>
-        </is>
-      </c>
-      <c r="C75" s="3" t="n"/>
-      <c r="D75" s="3" t="n"/>
-      <c r="E75" s="3" t="n"/>
-      <c r="F75" s="3" t="n"/>
-      <c r="G75" s="3" t="n"/>
-      <c r="H75" s="3" t="n"/>
-      <c r="I75" s="3" t="n"/>
-      <c r="J75" s="3" t="n"/>
-      <c r="K75" s="18">
-        <f>SUM(K72:K74)</f>
-        <v/>
-      </c>
-      <c r="L75" s="3" t="n"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="7" t="inlineStr">
-        <is>
-          <t>7.11</t>
-        </is>
-      </c>
-      <c r="B76" s="7" t="inlineStr">
-        <is>
-          <t>Twelve months defects liability and routine maintenance</t>
-        </is>
-      </c>
-      <c r="C76" s="7" t="n"/>
-      <c r="D76" s="7" t="n"/>
-      <c r="E76" s="7" t="n"/>
-      <c r="F76" s="7" t="n"/>
-      <c r="G76" s="7" t="n"/>
-      <c r="H76" s="7" t="n"/>
-      <c r="I76" s="7" t="n"/>
-      <c r="J76" s="7" t="n"/>
-      <c r="K76" s="7" t="n"/>
-      <c r="L76" s="7" t="n"/>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="I76" s="4" t="n"/>
+      <c r="J76" s="17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K76" s="4">
+        <f>IFERROR($G76*$I76,"")</f>
+        <v/>
+      </c>
+      <c r="L76" s="2" t="inlineStr">
+        <is>
+          <t>carried on past jobs</t>
+        </is>
+      </c>
     </row>
     <row r="77">
-      <c r="B77" s="14" t="inlineStr">
-        <is>
-          <t>Routine maintenance, 12 months</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>D-MAINT</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr"/>
-      <c r="E77" s="10" t="inlineStr">
-        <is>
-          <t>Bought in</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>ENGINEER</t>
-        </is>
-      </c>
-      <c r="G77" t="n">
-        <v>4</v>
-      </c>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>visit</t>
-        </is>
-      </c>
-      <c r="I77" s="4" t="n"/>
-      <c r="J77" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K77" s="4">
-        <f>IFERROR($G77*$I77,"")</f>
-        <v/>
-      </c>
-      <c r="L77" s="2" t="inlineStr">
-        <is>
-          <t>rate to be entered</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="B78" s="14" t="inlineStr">
-        <is>
-          <t>Contingency</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>D-CONT</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr"/>
-      <c r="E78" s="10" t="inlineStr">
-        <is>
-          <t>Bought in</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>ENGINEER</t>
-        </is>
-      </c>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>lot</t>
-        </is>
-      </c>
-      <c r="I78" s="4" t="n"/>
-      <c r="J78" s="17" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K78" s="4">
-        <f>IFERROR($G78*$I78,"")</f>
-        <v/>
-      </c>
-      <c r="L78" s="2" t="inlineStr">
-        <is>
-          <t>carried on past jobs</t>
-        </is>
-      </c>
+      <c r="A77" s="3" t="n"/>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>Section 7.11 total</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="n"/>
+      <c r="D77" s="3" t="n"/>
+      <c r="E77" s="3" t="n"/>
+      <c r="F77" s="3" t="n"/>
+      <c r="G77" s="3" t="n"/>
+      <c r="H77" s="3" t="n"/>
+      <c r="I77" s="3" t="n"/>
+      <c r="J77" s="3" t="n"/>
+      <c r="K77" s="18">
+        <f>SUM(K75:K76)</f>
+        <v/>
+      </c>
+      <c r="L77" s="3" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="3" t="n"/>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Section 7.11 total</t>
+          <t>TOTAL COST</t>
         </is>
       </c>
       <c r="C79" s="3" t="n"/>
@@ -3720,35 +3653,14 @@
       <c r="I79" s="3" t="n"/>
       <c r="J79" s="3" t="n"/>
       <c r="K79" s="18">
-        <f>SUM(K77:K78)</f>
+        <f>K9+K12+K15+K19+K22+K42+K57+K61+K68+K73+K77</f>
         <v/>
       </c>
       <c r="L79" s="3" t="n"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="3" t="n"/>
-      <c r="B81" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL COST</t>
-        </is>
-      </c>
-      <c r="C81" s="3" t="n"/>
-      <c r="D81" s="3" t="n"/>
-      <c r="E81" s="3" t="n"/>
-      <c r="F81" s="3" t="n"/>
-      <c r="G81" s="3" t="n"/>
-      <c r="H81" s="3" t="n"/>
-      <c r="I81" s="3" t="n"/>
-      <c r="J81" s="3" t="n"/>
-      <c r="K81" s="18">
-        <f>K9+K12+K15+K19+K22+K44+K59+K63+K70+K75+K79</f>
-        <v/>
-      </c>
-      <c r="L81" s="3" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="E46 E47 E48 E49 E50 E51 E52 E53 E54 E58 E61 E62 E65 E66 E67 E68 E72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E44 E45 E46 E47 E48 E49 E50 E51 E52 E56 E59 E60 E63 E64 E65 E66 E70" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"In-house,Subcontract"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3926,7 +3838,7 @@
         </is>
       </c>
       <c r="C7" s="4">
-        <f>Costing!K44</f>
+        <f>Costing!K42</f>
         <v/>
       </c>
       <c r="D7" s="17" t="n">
@@ -3949,7 +3861,7 @@
         </is>
       </c>
       <c r="C8" s="4">
-        <f>Costing!K59</f>
+        <f>Costing!K57</f>
         <v/>
       </c>
       <c r="D8" s="17" t="n">
@@ -3972,7 +3884,7 @@
         </is>
       </c>
       <c r="C9" s="4">
-        <f>Costing!K63</f>
+        <f>Costing!K61</f>
         <v/>
       </c>
       <c r="D9" s="17" t="n">
@@ -3995,7 +3907,7 @@
         </is>
       </c>
       <c r="C10" s="4">
-        <f>Costing!K70</f>
+        <f>Costing!K68</f>
         <v/>
       </c>
       <c r="D10" s="17" t="n">
@@ -4018,7 +3930,7 @@
         </is>
       </c>
       <c r="C11" s="4">
-        <f>Costing!K75</f>
+        <f>Costing!K73</f>
         <v/>
       </c>
       <c r="D11" s="17" t="n">
@@ -4041,7 +3953,7 @@
         </is>
       </c>
       <c r="C12" s="4">
-        <f>Costing!K79</f>
+        <f>Costing!K77</f>
         <v/>
       </c>
       <c r="D12" s="17" t="n">
@@ -4691,7 +4603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4911,7 +4823,7 @@
     <row r="14">
       <c r="B14" t="inlineStr">
         <is>
-          <t>65PN bolt set</t>
+          <t>65TE tube flange</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -4926,7 +4838,7 @@
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>65TE tube flange</t>
+          <t>65PN bolt set</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -4986,11 +4898,11 @@
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
-          <t>101mm tube pipe</t>
+          <t>Pipe insulation</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>12</v>
+        <v>219</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -5001,49 +4913,49 @@
     <row r="20">
       <c r="B20" t="inlineStr">
         <is>
-          <t>63mm tube pipe</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>12</v>
+          <t>Spare parts</t>
+        </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ea</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>Pipe insulation</t>
         </is>
       </c>
-      <c r="C21" t="n">
-        <v>243</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>m</t>
+      <c r="B21" s="7" t="n"/>
+      <c r="C21" s="7" t="n"/>
+      <c r="D21" s="7" t="n"/>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>insulation subcontractor — request a schedule of rates, $/m by diameter</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" t="inlineStr">
         <is>
-          <t>Spare parts</t>
-        </is>
+          <t>Pipe insulation</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>219</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>ea</t>
+          <t>m</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>Pipe insulation</t>
+          <t>Electrical power, control wiring and SCADA</t>
         </is>
       </c>
       <c r="B23" s="7" t="n"/>
@@ -5051,65 +4963,35 @@
       <c r="D23" s="7" t="n"/>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>insulation subcontractor — request a schedule of rates, $/m by diameter</t>
+          <t>electrical contractor — attach the Electrical tab</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" t="inlineStr">
         <is>
-          <t>Pipe insulation</t>
+          <t>Power and control wiring</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>243</v>
+        <v>1</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>lot</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>Electrical power, control wiring and SCADA</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="n"/>
-      <c r="C25" s="7" t="n"/>
-      <c r="D25" s="7" t="n"/>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>electrical contractor — attach the Electrical tab</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Power and control wiring</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>SCADA integration — Ignition</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
         <v>1</v>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>lot</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>SCADA integration — Ignition</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>lot</t>
         </is>
@@ -5376,7 +5258,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>65PN</t>
+          <t>65TE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -5409,7 +5291,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>65PN</t>
+          <t>65TE</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -5442,7 +5324,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>65TE</t>
+          <t>65PN</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -5475,7 +5357,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>65TE</t>
+          <t>65PN</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">

</xml_diff>